<commit_message>
Gemini: add test results for Cli (1-27, count: 26)
</commit_message>
<xml_diff>
--- a/Gemini-3.8-flash/summary.xlsx
+++ b/Gemini-3.8-flash/summary.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="row_type"/>
     <x:tableColumn id="2" name="round"/>
@@ -412,16 +412,16 @@
         <x:v>Results</x:v>
       </x:c>
       <x:c r="C6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$41,"Round1")</x:f>
-        <x:v>40</x:v>
+        <x:f>COUNTIF(Data!$B$2:$B$53,"Round1")</x:f>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$41,"Round2")</x:f>
+        <x:f>COUNTIF(Data!$B$2:$B$53,"Round2")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="11">
-        <x:f>COUNTA(Data!$C$2:$C$41)</x:f>
-        <x:v>40</x:v>
+        <x:f>COUNTA(Data!$C$2:$C$53)</x:f>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -435,16 +435,16 @@
         <x:v>Average line coverage</x:v>
       </x:c>
       <x:c r="C7" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$E$2:$E$41,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$41,"Round1",Data!$E$2:$E$41))</x:f>
-        <x:v>0.41775769230769233</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$E$2:$E$53,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$53,"Round1",Data!$E$2:$E$53))</x:f>
+        <x:v>0.2935594594594595</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$E$2:$E$41,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$41,"Round2",Data!$E$2:$E$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$E$2:$E$53,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$53,"Round2",Data!$E$2:$E$53))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E7" s="12">
-        <x:f>IF(COUNT(Data!$E$2:$E$41)=0,"",AVERAGE(Data!$E$2:$E$41))</x:f>
-        <x:v>0.41775769230769233</x:v>
+        <x:f>IF(COUNT(Data!$E$2:$E$53)=0,"",AVERAGE(Data!$E$2:$E$53))</x:f>
+        <x:v>0.2935594594594595</x:v>
       </x:c>
       <x:c r="F7" s="1"/>
       <x:c r="G7" s="1"/>
@@ -460,16 +460,16 @@
         </x:is>
       </x:c>
       <x:c r="C8" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$N$2:$N$41,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$41,"Round1",Data!$N$2:$N$41))</x:f>
-        <x:v>0.33461199999999997</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$N$2:$N$53,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$53,"Round1",Data!$N$2:$N$53))</x:f>
+        <x:v>0.23236944444444443</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$N$2:$N$41,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$41,"Round2",Data!$N$2:$N$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$N$2:$N$53,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$53,"Round2",Data!$N$2:$N$53))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E8" s="12">
-        <x:f>IF(COUNT(Data!$N$2:$N$41)=0,"",AVERAGE(Data!$N$2:$N$41))</x:f>
-        <x:v>0.33461199999999997</x:v>
+        <x:f>IF(COUNT(Data!$N$2:$N$53)=0,"",AVERAGE(Data!$N$2:$N$53))</x:f>
+        <x:v>0.23236944444444443</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -483,15 +483,15 @@
         <x:v>Revealing results</x:v>
       </x:c>
       <x:c r="C9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$41,"Round1",Data!$F$2:$F$41)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$53,"Round1",Data!$F$2:$F$53)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$41,"Round2",Data!$F$2:$F$41)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$53,"Round2",Data!$F$2:$F$53)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="11">
-        <x:f>SUM(Data!$F$2:$F$41)</x:f>
+        <x:f>SUM(Data!$F$2:$F$53)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="1"/>
@@ -529,16 +529,16 @@
         <x:v>Total tokens</x:v>
       </x:c>
       <x:c r="C11" s="10">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$G$2:$G$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round1",Data!$G$2:$G$41))</x:f>
-        <x:v>408508</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$G$2:$G$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$G$2:$G$53))</x:f>
+        <x:v>550016</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$G$2:$G$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round2",Data!$G$2:$G$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$G$2:$G$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$G$2:$G$53))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E11" s="11">
-        <x:f>IF(COUNT(Data!$G$2:$G$41)=0,"",SUM(Data!$G$2:$G$41))</x:f>
-        <x:v>408508</x:v>
+        <x:f>IF(COUNT(Data!$G$2:$G$53)=0,"",SUM(Data!$G$2:$G$53))</x:f>
+        <x:v>550016</x:v>
       </x:c>
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
@@ -552,16 +552,16 @@
         <x:v>Generation time (seconds)</x:v>
       </x:c>
       <x:c r="C12" s="6">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$H$2:$H$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round1",Data!$H$2:$H$41))</x:f>
-        <x:v>1699.67</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$H$2:$H$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$H$2:$H$53))</x:f>
+        <x:v>2288.59</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$H$2:$H$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round2",Data!$H$2:$H$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$H$2:$H$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$H$2:$H$53))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E12" s="13">
-        <x:f>IF(COUNT(Data!$H$2:$H$41)=0,"",SUM(Data!$H$2:$H$41))</x:f>
-        <x:v>1699.67</x:v>
+        <x:f>IF(COUNT(Data!$H$2:$H$53)=0,"",SUM(Data!$H$2:$H$53))</x:f>
+        <x:v>2288.59</x:v>
       </x:c>
       <x:c r="F12" s="1"/>
       <x:c r="G12" s="1"/>
@@ -575,16 +575,16 @@
         <x:v>Coverage records</x:v>
       </x:c>
       <x:c r="C13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$E$2:$E$41,"&lt;&gt;")</x:f>
-        <x:v>26</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$E$2:$E$53,"&lt;&gt;")</x:f>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$E$2:$E$41,"&lt;&gt;")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$E$2:$E$53,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="14">
-        <x:f>COUNT(Data!$E$2:$E$41)</x:f>
-        <x:v>26</x:v>
+        <x:f>COUNT(Data!$E$2:$E$53)</x:f>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="F13" s="1"/>
       <x:c r="G13" s="1"/>
@@ -600,16 +600,16 @@
         </x:is>
       </x:c>
       <x:c r="C14" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$J$2:$J$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round1",Data!$J$2:$J$41))</x:f>
-        <x:v>7946</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$J$2:$J$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$J$2:$J$53))</x:f>
+        <x:v>9047</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$J$2:$J$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round2",Data!$J$2:$J$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$J$2:$J$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$J$2:$J$53))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E14" s="4">
-        <x:f>IF(COUNT(Data!$J$2:$J$41)=0,"",SUM(Data!$J$2:$J$41))</x:f>
-        <x:v>7946</x:v>
+        <x:f>IF(COUNT(Data!$J$2:$J$53)=0,"",SUM(Data!$J$2:$J$53))</x:f>
+        <x:v>9047</x:v>
       </x:c>
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
@@ -625,15 +625,15 @@
         </x:is>
       </x:c>
       <x:c r="C15" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$K$2:$K$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round1",Data!$K$2:$K$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$K$2:$K$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$K$2:$K$53))</x:f>
         <x:v>4641</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$K$2:$K$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round2",Data!$K$2:$K$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$K$2:$K$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$K$2:$K$53))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E15" s="4">
-        <x:f>IF(COUNT(Data!$K$2:$K$41)=0,"",SUM(Data!$K$2:$K$41))</x:f>
+        <x:f>IF(COUNT(Data!$K$2:$K$53)=0,"",SUM(Data!$K$2:$K$53))</x:f>
         <x:v>4641</x:v>
       </x:c>
       <x:c r="F15" s="1"/>
@@ -650,16 +650,16 @@
         </x:is>
       </x:c>
       <x:c r="C16" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$L$2:$L$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round1",Data!$L$2:$L$41))</x:f>
-        <x:v>4011</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$L$2:$L$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$L$2:$L$53))</x:f>
+        <x:v>4611</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$L$2:$L$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round2",Data!$L$2:$L$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$L$2:$L$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$L$2:$L$53))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E16" s="4">
-        <x:f>IF(COUNT(Data!$L$2:$L$41)=0,"",SUM(Data!$L$2:$L$41))</x:f>
-        <x:v>4011</x:v>
+        <x:f>IF(COUNT(Data!$L$2:$L$53)=0,"",SUM(Data!$L$2:$L$53))</x:f>
+        <x:v>4611</x:v>
       </x:c>
       <x:c r="F16" s="1"/>
       <x:c r="G16" s="1"/>
@@ -675,15 +675,15 @@
         </x:is>
       </x:c>
       <x:c r="C17" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$M$2:$M$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round1",Data!$M$2:$M$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$M$2:$M$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$M$2:$M$53))</x:f>
         <x:v>1820</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$M$2:$M$41,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$41,"Round2",Data!$M$2:$M$41))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$M$2:$M$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$M$2:$M$53))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E17" s="4">
-        <x:f>IF(COUNT(Data!$M$2:$M$41)=0,"",SUM(Data!$M$2:$M$41))</x:f>
+        <x:f>IF(COUNT(Data!$M$2:$M$53)=0,"",SUM(Data!$M$2:$M$53))</x:f>
         <x:v>1820</x:v>
       </x:c>
       <x:c r="F17" s="1"/>
@@ -718,15 +718,15 @@
         <x:v>REVEALING</x:v>
       </x:c>
       <x:c r="C19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$D$2:$D$41,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$D$2:$D$53,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$D$2:$D$41,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$D$2:$D$53,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$41,"REVEALING")</x:f>
+        <x:f>COUNTIF(Data!$D$2:$D$53,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="1"/>
@@ -741,15 +741,15 @@
         <x:v>NOT_REVEALING</x:v>
       </x:c>
       <x:c r="C20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$D$2:$D$41,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$D$2:$D$53,"NOT_REVEALING")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$D$2:$D$41,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$D$2:$D$53,"NOT_REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E20" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$41,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIF(Data!$D$2:$D$53,"NOT_REVEALING")</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="F20" s="1"/>
@@ -764,16 +764,16 @@
         <x:v>NOT_AVAILABLE</x:v>
       </x:c>
       <x:c r="C21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$D$2:$D$41,"NOT_AVAILABLE")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$D$2:$D$53,"NOT_AVAILABLE")</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$D$2:$D$41,"NOT_AVAILABLE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$D$2:$D$53,"NOT_AVAILABLE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$41,"NOT_AVAILABLE")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$53,"NOT_AVAILABLE")</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F21" s="1"/>
       <x:c r="G21" s="1"/>
@@ -787,16 +787,16 @@
         <x:v>INCONCLUSIVE</x:v>
       </x:c>
       <x:c r="C22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round1",Data!$D$2:$D$41,"INCONCLUSIVE")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$D$2:$D$53,"INCONCLUSIVE")</x:f>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$41,"Round2",Data!$D$2:$D$41,"INCONCLUSIVE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$D$2:$D$53,"INCONCLUSIVE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$41,"INCONCLUSIVE")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$53,"INCONCLUSIVE")</x:f>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F22" s="1"/>
       <x:c r="G22" s="1"/>
@@ -836,7 +836,7 @@
       <x:c r="A25" s="1"/>
       <x:c r="B25" s="3" t="inlineStr">
         <x:is>
-          <x:t>Updated: 2026-09-30 05:25:08 +0700</x:t>
+          <x:t>Updated: 2026-09-30 05:25:49 +0700</x:t>
         </x:is>
       </x:c>
       <x:c r="C25" s="3"/>
@@ -2466,32 +2466,44 @@
       </x:c>
       <x:c r="C34" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_16</x:t>
+          <x:t>Cli_15</x:t>
         </x:is>
       </x:c>
       <x:c r="D34" s="1" t="inlineStr">
         <x:is>
-          <x:t>NOT_AVAILABLE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E34" s="5"/>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E34" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
       <x:c r="F34" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G34" s="4">
-        <x:v>46594</x:v>
+        <x:v>13614</x:v>
       </x:c>
       <x:c r="H34" s="6">
-        <x:v>205.57</x:v>
+        <x:v>62.19</x:v>
       </x:c>
       <x:c r="I34" s="16">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J34" s="0"/>
-      <x:c r="K34" s="4"/>
-      <x:c r="L34" s="4"/>
-      <x:c r="M34" s="4"/>
-      <x:c r="N34" s="5"/>
+      <x:c r="J34" s="0">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="K34" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L34" s="4">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="M34" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N34" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="1" t="inlineStr">
@@ -2506,44 +2518,32 @@
       </x:c>
       <x:c r="C35" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_2</x:t>
+          <x:t>Cli_16</x:t>
         </x:is>
       </x:c>
       <x:c r="D35" s="1" t="inlineStr">
         <x:is>
-          <x:t>INCONCLUSIVE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E35" s="5">
-        <x:v>0.0</x:v>
-      </x:c>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E35" s="5"/>
       <x:c r="F35" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G35" s="4">
-        <x:v>10030</x:v>
+        <x:v>46594</x:v>
       </x:c>
       <x:c r="H35" s="6">
-        <x:v>37.59</x:v>
+        <x:v>205.57</x:v>
       </x:c>
       <x:c r="I35" s="16">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J35" s="0">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="K35" s="4">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L35" s="4">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="M35" s="4">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N35" s="5">
-        <x:v>0.0</x:v>
-      </x:c>
+      <x:c r="J35" s="0"/>
+      <x:c r="K35" s="4"/>
+      <x:c r="L35" s="4"/>
+      <x:c r="M35" s="4"/>
+      <x:c r="N35" s="5"/>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
       <x:c r="A36" s="1" t="inlineStr">
@@ -2558,7 +2558,7 @@
       </x:c>
       <x:c r="C36" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_3</x:t>
+          <x:t>Cli_17</x:t>
         </x:is>
       </x:c>
       <x:c r="D36" s="1" t="inlineStr">
@@ -2573,22 +2573,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G36" s="4">
-        <x:v>7513</x:v>
+        <x:v>9139</x:v>
       </x:c>
       <x:c r="H36" s="6">
-        <x:v>29.89</x:v>
+        <x:v>33.38</x:v>
       </x:c>
       <x:c r="I36" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J36" s="0">
-        <x:v>55</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="K36" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L36" s="4">
-        <x:v>20</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M36" s="4">
         <x:v>0</x:v>
@@ -2610,7 +2610,7 @@
       </x:c>
       <x:c r="C37" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_4</x:t>
+          <x:t>Cli_18</x:t>
         </x:is>
       </x:c>
       <x:c r="D37" s="1" t="inlineStr">
@@ -2625,22 +2625,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G37" s="4">
-        <x:v>9748</x:v>
+        <x:v>8138</x:v>
       </x:c>
       <x:c r="H37" s="6">
-        <x:v>32.15</x:v>
+        <x:v>36.55</x:v>
       </x:c>
       <x:c r="I37" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J37" s="0">
-        <x:v>99</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="K37" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L37" s="4">
-        <x:v>68</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M37" s="4">
         <x:v>0</x:v>
@@ -2662,7 +2662,7 @@
       </x:c>
       <x:c r="C38" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_5</x:t>
+          <x:t>Cli_19</x:t>
         </x:is>
       </x:c>
       <x:c r="D38" s="1" t="inlineStr">
@@ -2677,22 +2677,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G38" s="4">
-        <x:v>4221</x:v>
+        <x:v>6904</x:v>
       </x:c>
       <x:c r="H38" s="6">
-        <x:v>17.32</x:v>
+        <x:v>47.91</x:v>
       </x:c>
       <x:c r="I38" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J38" s="0">
-        <x:v>11</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="K38" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L38" s="4">
-        <x:v>8</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M38" s="4">
         <x:v>0</x:v>
@@ -2714,7 +2714,7 @@
       </x:c>
       <x:c r="C39" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_7</x:t>
+          <x:t>Cli_2</x:t>
         </x:is>
       </x:c>
       <x:c r="D39" s="1" t="inlineStr">
@@ -2729,10 +2729,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G39" s="4">
-        <x:v>6282</x:v>
+        <x:v>10030</x:v>
       </x:c>
       <x:c r="H39" s="6">
-        <x:v>23.46</x:v>
+        <x:v>37.59</x:v>
       </x:c>
       <x:c r="I39" s="16">
         <x:v>1</x:v>
@@ -2744,7 +2744,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L39" s="4">
-        <x:v>27</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M39" s="4">
         <x:v>0</x:v>
@@ -2766,7 +2766,7 @@
       </x:c>
       <x:c r="C40" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_8</x:t>
+          <x:t>Cli_20</x:t>
         </x:is>
       </x:c>
       <x:c r="D40" s="1" t="inlineStr">
@@ -2781,22 +2781,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G40" s="4">
-        <x:v>10601</x:v>
+        <x:v>9235</x:v>
       </x:c>
       <x:c r="H40" s="6">
-        <x:v>36.83</x:v>
+        <x:v>33.36</x:v>
       </x:c>
       <x:c r="I40" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J40" s="0">
-        <x:v>192</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="K40" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L40" s="4">
-        <x:v>104</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="M40" s="4">
         <x:v>0</x:v>
@@ -2818,42 +2818,654 @@
       </x:c>
       <x:c r="C41" s="1" t="inlineStr">
         <x:is>
+          <x:t>Cli_21</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D41" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E41" s="5"/>
+      <x:c r="F41" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G41" s="4">
+        <x:v>44499</x:v>
+      </x:c>
+      <x:c r="H41" s="6">
+        <x:v>193.42</x:v>
+      </x:c>
+      <x:c r="I41" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J41" s="0"/>
+      <x:c r="K41" s="4"/>
+      <x:c r="L41" s="4"/>
+      <x:c r="M41" s="4"/>
+      <x:c r="N41" s="5"/>
+    </x:row>
+    <x:row r="42" ht="24" customHeight="1">
+      <x:c r="A42" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B42" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D42" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E42" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F42" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G42" s="4">
+        <x:v>8943</x:v>
+      </x:c>
+      <x:c r="H42" s="6">
+        <x:v>33.33</x:v>
+      </x:c>
+      <x:c r="I42" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J42" s="0">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="K42" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L42" s="4">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="M42" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N42" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="24" customHeight="1">
+      <x:c r="A43" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B43" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_23</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D43" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E43" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F43" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G43" s="4">
+        <x:v>8536</x:v>
+      </x:c>
+      <x:c r="H43" s="6">
+        <x:v>23.62</x:v>
+      </x:c>
+      <x:c r="I43" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J43" s="0">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="K43" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L43" s="4">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="M43" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N43" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="24" customHeight="1">
+      <x:c r="A44" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B44" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C44" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_24</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D44" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E44" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F44" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G44" s="4">
+        <x:v>9526</x:v>
+      </x:c>
+      <x:c r="H44" s="6">
+        <x:v>31.4</x:v>
+      </x:c>
+      <x:c r="I44" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J44" s="0">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="K44" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L44" s="4">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="M44" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N44" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="24" customHeight="1">
+      <x:c r="A45" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B45" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C45" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_25</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D45" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E45" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F45" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G45" s="4">
+        <x:v>10582</x:v>
+      </x:c>
+      <x:c r="H45" s="6">
+        <x:v>36.88</x:v>
+      </x:c>
+      <x:c r="I45" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J45" s="0">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="K45" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L45" s="4">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="M45" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N45" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="24" customHeight="1">
+      <x:c r="A46" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B46" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C46" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_26</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D46" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E46" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F46" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G46" s="4">
+        <x:v>7169</x:v>
+      </x:c>
+      <x:c r="H46" s="6">
+        <x:v>36.27</x:v>
+      </x:c>
+      <x:c r="I46" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J46" s="0">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="K46" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L46" s="4">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="M46" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N46" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="24" customHeight="1">
+      <x:c r="A47" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B47" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C47" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_27</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D47" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E47" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F47" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G47" s="4">
+        <x:v>5223</x:v>
+      </x:c>
+      <x:c r="H47" s="6">
+        <x:v>20.61</x:v>
+      </x:c>
+      <x:c r="I47" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J47" s="0">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="K47" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L47" s="4">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="M47" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N47" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="24" customHeight="1">
+      <x:c r="A48" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B48" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C48" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D48" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E48" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F48" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G48" s="4">
+        <x:v>7513</x:v>
+      </x:c>
+      <x:c r="H48" s="6">
+        <x:v>29.89</x:v>
+      </x:c>
+      <x:c r="I48" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J48" s="0">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="K48" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L48" s="4">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="M48" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N48" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="24" customHeight="1">
+      <x:c r="A49" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B49" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C49" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D49" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E49" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F49" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G49" s="4">
+        <x:v>9748</x:v>
+      </x:c>
+      <x:c r="H49" s="6">
+        <x:v>32.15</x:v>
+      </x:c>
+      <x:c r="I49" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J49" s="0">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="K49" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L49" s="4">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="M49" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N49" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="24" customHeight="1">
+      <x:c r="A50" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B50" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C50" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D50" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E50" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F50" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G50" s="4">
+        <x:v>4221</x:v>
+      </x:c>
+      <x:c r="H50" s="6">
+        <x:v>17.32</x:v>
+      </x:c>
+      <x:c r="I50" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J50" s="0">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="K50" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L50" s="4">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="M50" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N50" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="24" customHeight="1">
+      <x:c r="A51" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B51" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C51" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D51" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E51" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F51" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G51" s="4">
+        <x:v>6282</x:v>
+      </x:c>
+      <x:c r="H51" s="6">
+        <x:v>23.46</x:v>
+      </x:c>
+      <x:c r="I51" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J51" s="0">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="K51" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L51" s="4">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="M51" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N51" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="24" customHeight="1">
+      <x:c r="A52" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B52" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C52" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D52" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E52" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F52" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G52" s="4">
+        <x:v>10601</x:v>
+      </x:c>
+      <x:c r="H52" s="6">
+        <x:v>36.83</x:v>
+      </x:c>
+      <x:c r="I52" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J52" s="0">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="K52" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L52" s="4">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="M52" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N52" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="24" customHeight="1">
+      <x:c r="A53" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B53" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C53" s="1" t="inlineStr">
+        <x:is>
           <x:t>Cli_9</x:t>
         </x:is>
       </x:c>
-      <x:c r="D41" s="1" t="inlineStr">
+      <x:c r="D53" s="1" t="inlineStr">
         <x:is>
           <x:t>INCONCLUSIVE</x:t>
         </x:is>
       </x:c>
-      <x:c r="E41" s="5">
-        <x:v>0.0</x:v>
-      </x:c>
-      <x:c r="F41" s="4">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G41" s="4">
+      <x:c r="E53" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F53" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G53" s="4">
         <x:v>12531</x:v>
       </x:c>
-      <x:c r="H41" s="6">
+      <x:c r="H53" s="6">
         <x:v>50.14</x:v>
       </x:c>
-      <x:c r="I41" s="16">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J41" s="0">
+      <x:c r="I53" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J53" s="0">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="K41" s="4">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L41" s="4">
+      <x:c r="K53" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L53" s="4">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="M41" s="4">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N41" s="5">
+      <x:c r="M53" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N53" s="5">
         <x:v>0.0</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Gemini: add test results for Cli (28-40, count: 13), Closure (1-12, count: 12)
</commit_message>
<xml_diff>
--- a/Gemini-3.8-flash/summary.xlsx
+++ b/Gemini-3.8-flash/summary.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="row_type"/>
     <x:tableColumn id="2" name="round"/>
@@ -412,16 +412,16 @@
         <x:v>Results</x:v>
       </x:c>
       <x:c r="C6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$53,"Round1")</x:f>
-        <x:v>52</x:v>
+        <x:f>COUNTIF(Data!$B$2:$B$78,"Round1")</x:f>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$53,"Round2")</x:f>
+        <x:f>COUNTIF(Data!$B$2:$B$78,"Round2")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="11">
-        <x:f>COUNTA(Data!$C$2:$C$53)</x:f>
-        <x:v>52</x:v>
+        <x:f>COUNTA(Data!$C$2:$C$78)</x:f>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -435,16 +435,16 @@
         <x:v>Average line coverage</x:v>
       </x:c>
       <x:c r="C7" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$E$2:$E$53,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$53,"Round1",Data!$E$2:$E$53))</x:f>
-        <x:v>0.2935594594594595</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$E$2:$E$78,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$78,"Round1",Data!$E$2:$E$78))</x:f>
+        <x:v>0.3495192307692308</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$E$2:$E$53,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$53,"Round2",Data!$E$2:$E$53))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$E$2:$E$78,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$78,"Round2",Data!$E$2:$E$78))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E7" s="12">
-        <x:f>IF(COUNT(Data!$E$2:$E$53)=0,"",AVERAGE(Data!$E$2:$E$53))</x:f>
-        <x:v>0.2935594594594595</x:v>
+        <x:f>IF(COUNT(Data!$E$2:$E$78)=0,"",AVERAGE(Data!$E$2:$E$78))</x:f>
+        <x:v>0.3495192307692308</x:v>
       </x:c>
       <x:c r="F7" s="1"/>
       <x:c r="G7" s="1"/>
@@ -460,16 +460,16 @@
         </x:is>
       </x:c>
       <x:c r="C8" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$N$2:$N$53,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$53,"Round1",Data!$N$2:$N$53))</x:f>
-        <x:v>0.23236944444444443</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$N$2:$N$78,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$78,"Round1",Data!$N$2:$N$78))</x:f>
+        <x:v>0.2913882352941176</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$N$2:$N$53,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$53,"Round2",Data!$N$2:$N$53))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$N$2:$N$78,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$78,"Round2",Data!$N$2:$N$78))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E8" s="12">
-        <x:f>IF(COUNT(Data!$N$2:$N$53)=0,"",AVERAGE(Data!$N$2:$N$53))</x:f>
-        <x:v>0.23236944444444443</x:v>
+        <x:f>IF(COUNT(Data!$N$2:$N$78)=0,"",AVERAGE(Data!$N$2:$N$78))</x:f>
+        <x:v>0.2913882352941176</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -483,15 +483,15 @@
         <x:v>Revealing results</x:v>
       </x:c>
       <x:c r="C9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$53,"Round1",Data!$F$2:$F$53)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$78,"Round1",Data!$F$2:$F$78)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$53,"Round2",Data!$F$2:$F$53)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$78,"Round2",Data!$F$2:$F$78)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="11">
-        <x:f>SUM(Data!$F$2:$F$53)</x:f>
+        <x:f>SUM(Data!$F$2:$F$78)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="1"/>
@@ -529,16 +529,16 @@
         <x:v>Total tokens</x:v>
       </x:c>
       <x:c r="C11" s="10">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$G$2:$G$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$G$2:$G$53))</x:f>
-        <x:v>550016</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$G$2:$G$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$G$2:$G$78))</x:f>
+        <x:v>821823</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$G$2:$G$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$G$2:$G$53))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$G$2:$G$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$G$2:$G$78))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E11" s="11">
-        <x:f>IF(COUNT(Data!$G$2:$G$53)=0,"",SUM(Data!$G$2:$G$53))</x:f>
-        <x:v>550016</x:v>
+        <x:f>IF(COUNT(Data!$G$2:$G$78)=0,"",SUM(Data!$G$2:$G$78))</x:f>
+        <x:v>821823</x:v>
       </x:c>
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
@@ -552,16 +552,16 @@
         <x:v>Generation time (seconds)</x:v>
       </x:c>
       <x:c r="C12" s="6">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$H$2:$H$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$H$2:$H$53))</x:f>
-        <x:v>2288.59</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$H$2:$H$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$H$2:$H$78))</x:f>
+        <x:v>3210.91</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$H$2:$H$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$H$2:$H$53))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$H$2:$H$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$H$2:$H$78))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E12" s="13">
-        <x:f>IF(COUNT(Data!$H$2:$H$53)=0,"",SUM(Data!$H$2:$H$53))</x:f>
-        <x:v>2288.59</x:v>
+        <x:f>IF(COUNT(Data!$H$2:$H$78)=0,"",SUM(Data!$H$2:$H$78))</x:f>
+        <x:v>3210.91</x:v>
       </x:c>
       <x:c r="F12" s="1"/>
       <x:c r="G12" s="1"/>
@@ -575,16 +575,16 @@
         <x:v>Coverage records</x:v>
       </x:c>
       <x:c r="C13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$E$2:$E$53,"&lt;&gt;")</x:f>
-        <x:v>37</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$E$2:$E$78,"&lt;&gt;")</x:f>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$E$2:$E$53,"&lt;&gt;")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$E$2:$E$78,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="14">
-        <x:f>COUNT(Data!$E$2:$E$53)</x:f>
-        <x:v>37</x:v>
+        <x:f>COUNT(Data!$E$2:$E$78)</x:f>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="F13" s="1"/>
       <x:c r="G13" s="1"/>
@@ -600,16 +600,16 @@
         </x:is>
       </x:c>
       <x:c r="C14" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$J$2:$J$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$J$2:$J$53))</x:f>
-        <x:v>9047</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$J$2:$J$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$J$2:$J$78))</x:f>
+        <x:v>11941</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$J$2:$J$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$J$2:$J$53))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$J$2:$J$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$J$2:$J$78))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E14" s="4">
-        <x:f>IF(COUNT(Data!$J$2:$J$53)=0,"",SUM(Data!$J$2:$J$53))</x:f>
-        <x:v>9047</x:v>
+        <x:f>IF(COUNT(Data!$J$2:$J$78)=0,"",SUM(Data!$J$2:$J$78))</x:f>
+        <x:v>11941</x:v>
       </x:c>
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
@@ -625,16 +625,16 @@
         </x:is>
       </x:c>
       <x:c r="C15" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$K$2:$K$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$K$2:$K$53))</x:f>
-        <x:v>4641</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$K$2:$K$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$K$2:$K$78))</x:f>
+        <x:v>5813</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$K$2:$K$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$K$2:$K$53))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$K$2:$K$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$K$2:$K$78))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E15" s="4">
-        <x:f>IF(COUNT(Data!$K$2:$K$53)=0,"",SUM(Data!$K$2:$K$53))</x:f>
-        <x:v>4641</x:v>
+        <x:f>IF(COUNT(Data!$K$2:$K$78)=0,"",SUM(Data!$K$2:$K$78))</x:f>
+        <x:v>5813</x:v>
       </x:c>
       <x:c r="F15" s="1"/>
       <x:c r="G15" s="1"/>
@@ -650,16 +650,16 @@
         </x:is>
       </x:c>
       <x:c r="C16" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$L$2:$L$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$L$2:$L$53))</x:f>
-        <x:v>4611</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$L$2:$L$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$L$2:$L$78))</x:f>
+        <x:v>6480</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$L$2:$L$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$L$2:$L$53))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$L$2:$L$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$L$2:$L$78))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E16" s="4">
-        <x:f>IF(COUNT(Data!$L$2:$L$53)=0,"",SUM(Data!$L$2:$L$53))</x:f>
-        <x:v>4611</x:v>
+        <x:f>IF(COUNT(Data!$L$2:$L$78)=0,"",SUM(Data!$L$2:$L$78))</x:f>
+        <x:v>6480</x:v>
       </x:c>
       <x:c r="F16" s="1"/>
       <x:c r="G16" s="1"/>
@@ -675,16 +675,16 @@
         </x:is>
       </x:c>
       <x:c r="C17" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$M$2:$M$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round1",Data!$M$2:$M$53))</x:f>
-        <x:v>1820</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$M$2:$M$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$M$2:$M$78))</x:f>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$M$2:$M$53,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$53,"Round2",Data!$M$2:$M$53))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$M$2:$M$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$M$2:$M$78))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E17" s="4">
-        <x:f>IF(COUNT(Data!$M$2:$M$53)=0,"",SUM(Data!$M$2:$M$53))</x:f>
-        <x:v>1820</x:v>
+        <x:f>IF(COUNT(Data!$M$2:$M$78)=0,"",SUM(Data!$M$2:$M$78))</x:f>
+        <x:v>2409</x:v>
       </x:c>
       <x:c r="F17" s="1"/>
       <x:c r="G17" s="1"/>
@@ -718,15 +718,15 @@
         <x:v>REVEALING</x:v>
       </x:c>
       <x:c r="C19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$D$2:$D$53,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$D$2:$D$78,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$D$2:$D$53,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$D$2:$D$78,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$53,"REVEALING")</x:f>
+        <x:f>COUNTIF(Data!$D$2:$D$78,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="1"/>
@@ -741,16 +741,16 @@
         <x:v>NOT_REVEALING</x:v>
       </x:c>
       <x:c r="C20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$D$2:$D$53,"NOT_REVEALING")</x:f>
-        <x:v>12</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$D$2:$D$78,"NOT_REVEALING")</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$D$2:$D$53,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$D$2:$D$78,"NOT_REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E20" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$53,"NOT_REVEALING")</x:f>
-        <x:v>12</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$78,"NOT_REVEALING")</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F20" s="1"/>
       <x:c r="G20" s="1"/>
@@ -764,16 +764,16 @@
         <x:v>NOT_AVAILABLE</x:v>
       </x:c>
       <x:c r="C21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$D$2:$D$53,"NOT_AVAILABLE")</x:f>
-        <x:v>15</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$D$2:$D$78,"NOT_AVAILABLE")</x:f>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$D$2:$D$53,"NOT_AVAILABLE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$D$2:$D$78,"NOT_AVAILABLE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$53,"NOT_AVAILABLE")</x:f>
-        <x:v>15</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$78,"NOT_AVAILABLE")</x:f>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F21" s="1"/>
       <x:c r="G21" s="1"/>
@@ -787,16 +787,16 @@
         <x:v>INCONCLUSIVE</x:v>
       </x:c>
       <x:c r="C22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round1",Data!$D$2:$D$53,"INCONCLUSIVE")</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$D$2:$D$78,"INCONCLUSIVE")</x:f>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$53,"Round2",Data!$D$2:$D$53,"INCONCLUSIVE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$D$2:$D$78,"INCONCLUSIVE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$53,"INCONCLUSIVE")</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$78,"INCONCLUSIVE")</x:f>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F22" s="1"/>
       <x:c r="G22" s="1"/>
@@ -836,7 +836,7 @@
       <x:c r="A25" s="1"/>
       <x:c r="B25" s="3" t="inlineStr">
         <x:is>
-          <x:t>Updated: 2026-09-30 05:25:49 +0700</x:t>
+          <x:t>Updated: 2026-09-30 05:32:32 +0700</x:t>
         </x:is>
       </x:c>
       <x:c r="C25" s="3"/>
@@ -3170,7 +3170,7 @@
       </x:c>
       <x:c r="C48" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_3</x:t>
+          <x:t>Cli_28</x:t>
         </x:is>
       </x:c>
       <x:c r="D48" s="1" t="inlineStr">
@@ -3185,22 +3185,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G48" s="4">
-        <x:v>7513</x:v>
+        <x:v>15637</x:v>
       </x:c>
       <x:c r="H48" s="6">
-        <x:v>29.89</x:v>
+        <x:v>65.89</x:v>
       </x:c>
       <x:c r="I48" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J48" s="0">
-        <x:v>55</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="K48" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L48" s="4">
-        <x:v>20</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="M48" s="4">
         <x:v>0</x:v>
@@ -3222,7 +3222,7 @@
       </x:c>
       <x:c r="C49" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_4</x:t>
+          <x:t>Cli_29</x:t>
         </x:is>
       </x:c>
       <x:c r="D49" s="1" t="inlineStr">
@@ -3237,22 +3237,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G49" s="4">
-        <x:v>9748</x:v>
+        <x:v>4304</x:v>
       </x:c>
       <x:c r="H49" s="6">
-        <x:v>32.15</x:v>
+        <x:v>15.98</x:v>
       </x:c>
       <x:c r="I49" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J49" s="0">
-        <x:v>99</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="K49" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L49" s="4">
-        <x:v>68</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="M49" s="4">
         <x:v>0</x:v>
@@ -3274,7 +3274,7 @@
       </x:c>
       <x:c r="C50" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_5</x:t>
+          <x:t>Cli_3</x:t>
         </x:is>
       </x:c>
       <x:c r="D50" s="1" t="inlineStr">
@@ -3289,22 +3289,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G50" s="4">
-        <x:v>4221</x:v>
+        <x:v>7513</x:v>
       </x:c>
       <x:c r="H50" s="6">
-        <x:v>17.32</x:v>
+        <x:v>29.89</x:v>
       </x:c>
       <x:c r="I50" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J50" s="0">
-        <x:v>11</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="K50" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L50" s="4">
-        <x:v>8</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="M50" s="4">
         <x:v>0</x:v>
@@ -3326,7 +3326,7 @@
       </x:c>
       <x:c r="C51" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_7</x:t>
+          <x:t>Cli_30</x:t>
         </x:is>
       </x:c>
       <x:c r="D51" s="1" t="inlineStr">
@@ -3341,22 +3341,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G51" s="4">
-        <x:v>6282</x:v>
+        <x:v>21749</x:v>
       </x:c>
       <x:c r="H51" s="6">
-        <x:v>23.46</x:v>
+        <x:v>79.29</x:v>
       </x:c>
       <x:c r="I51" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J51" s="0">
-        <x:v>68</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="K51" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L51" s="4">
-        <x:v>27</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="M51" s="4">
         <x:v>0</x:v>
@@ -3378,7 +3378,7 @@
       </x:c>
       <x:c r="C52" s="1" t="inlineStr">
         <x:is>
-          <x:t>Cli_8</x:t>
+          <x:t>Cli_31</x:t>
         </x:is>
       </x:c>
       <x:c r="D52" s="1" t="inlineStr">
@@ -3393,22 +3393,22 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G52" s="4">
-        <x:v>10601</x:v>
+        <x:v>35718</x:v>
       </x:c>
       <x:c r="H52" s="6">
-        <x:v>36.83</x:v>
+        <x:v>128.01</x:v>
       </x:c>
       <x:c r="I52" s="16">
         <x:v>1</x:v>
       </x:c>
       <x:c r="J52" s="0">
-        <x:v>192</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="K52" s="4">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L52" s="4">
-        <x:v>104</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="M52" s="4">
         <x:v>0</x:v>
@@ -3430,44 +3430,1192 @@
       </x:c>
       <x:c r="C53" s="1" t="inlineStr">
         <x:is>
+          <x:t>Cli_32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D53" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E53" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F53" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G53" s="4">
+        <x:v>11747</x:v>
+      </x:c>
+      <x:c r="H53" s="6">
+        <x:v>39.7</x:v>
+      </x:c>
+      <x:c r="I53" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J53" s="0">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="K53" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L53" s="4">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="M53" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N53" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="24" customHeight="1">
+      <x:c r="A54" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B54" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C54" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_33</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D54" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E54" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F54" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G54" s="4">
+        <x:v>11599</x:v>
+      </x:c>
+      <x:c r="H54" s="6">
+        <x:v>38.46</x:v>
+      </x:c>
+      <x:c r="I54" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J54" s="0">
+        <x:v>201</x:v>
+      </x:c>
+      <x:c r="K54" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L54" s="4">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="M54" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N54" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="24" customHeight="1">
+      <x:c r="A55" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B55" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C55" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_34</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D55" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E55" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F55" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G55" s="4">
+        <x:v>20618</x:v>
+      </x:c>
+      <x:c r="H55" s="6">
+        <x:v>69.37</x:v>
+      </x:c>
+      <x:c r="I55" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J55" s="0">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="K55" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L55" s="4">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="M55" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N55" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="24" customHeight="1">
+      <x:c r="A56" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B56" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C56" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_35</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D56" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E56" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="F56" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G56" s="4">
+        <x:v>7863</x:v>
+      </x:c>
+      <x:c r="H56" s="6">
+        <x:v>27.08</x:v>
+      </x:c>
+      <x:c r="I56" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J56" s="0">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="K56" s="4">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="L56" s="4">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="M56" s="4">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="N56" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="24" customHeight="1">
+      <x:c r="A57" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B57" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C57" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_36</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D57" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_REVEALING</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E57" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="F57" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G57" s="4">
+        <x:v>13646</x:v>
+      </x:c>
+      <x:c r="H57" s="6">
+        <x:v>53.17</x:v>
+      </x:c>
+      <x:c r="I57" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J57" s="0">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="K57" s="4">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="L57" s="4">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="M57" s="4">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="N57" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="24" customHeight="1">
+      <x:c r="A58" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B58" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C58" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_37</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D58" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_REVEALING</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E58" s="5">
+        <x:v>0.9571999999999999</x:v>
+      </x:c>
+      <x:c r="F58" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G58" s="4">
+        <x:v>11683</x:v>
+      </x:c>
+      <x:c r="H58" s="6">
+        <x:v>44.57</x:v>
+      </x:c>
+      <x:c r="I58" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J58" s="0">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="K58" s="4">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="L58" s="4">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="M58" s="4">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="N58" s="5">
+        <x:v>0.8418000000000001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="24" customHeight="1">
+      <x:c r="A59" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B59" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C59" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_38</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D59" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E59" s="5">
+        <x:v>0.9372</x:v>
+      </x:c>
+      <x:c r="F59" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G59" s="4">
+        <x:v>16777</x:v>
+      </x:c>
+      <x:c r="H59" s="6">
+        <x:v>74.76</x:v>
+      </x:c>
+      <x:c r="I59" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J59" s="0">
+        <x:v>191</x:v>
+      </x:c>
+      <x:c r="K59" s="4">
+        <x:v>179</x:v>
+      </x:c>
+      <x:c r="L59" s="4">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="M59" s="4">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="N59" s="5">
+        <x:v>0.8354</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="24" customHeight="1">
+      <x:c r="A60" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B60" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C60" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_39</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D60" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E60" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="F60" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G60" s="4">
+        <x:v>6785</x:v>
+      </x:c>
+      <x:c r="H60" s="6">
+        <x:v>25.02</x:v>
+      </x:c>
+      <x:c r="I60" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J60" s="0">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="K60" s="4">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="L60" s="4">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="M60" s="4">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="N60" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="24" customHeight="1">
+      <x:c r="A61" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B61" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C61" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D61" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E61" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F61" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G61" s="4">
+        <x:v>9748</x:v>
+      </x:c>
+      <x:c r="H61" s="6">
+        <x:v>32.15</x:v>
+      </x:c>
+      <x:c r="I61" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J61" s="0">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="K61" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L61" s="4">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="M61" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N61" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="24" customHeight="1">
+      <x:c r="A62" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B62" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C62" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_40</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D62" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E62" s="5"/>
+      <x:c r="F62" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G62" s="4">
+        <x:v>7021</x:v>
+      </x:c>
+      <x:c r="H62" s="6">
+        <x:v>24.33</x:v>
+      </x:c>
+      <x:c r="I62" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J62" s="0"/>
+      <x:c r="K62" s="4"/>
+      <x:c r="L62" s="4"/>
+      <x:c r="M62" s="4"/>
+      <x:c r="N62" s="5"/>
+    </x:row>
+    <x:row r="63" ht="24" customHeight="1">
+      <x:c r="A63" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B63" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C63" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D63" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E63" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F63" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G63" s="4">
+        <x:v>4221</x:v>
+      </x:c>
+      <x:c r="H63" s="6">
+        <x:v>17.32</x:v>
+      </x:c>
+      <x:c r="I63" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J63" s="0">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="K63" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L63" s="4">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="M63" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N63" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="24" customHeight="1">
+      <x:c r="A64" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B64" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C64" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D64" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E64" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F64" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G64" s="4">
+        <x:v>6282</x:v>
+      </x:c>
+      <x:c r="H64" s="6">
+        <x:v>23.46</x:v>
+      </x:c>
+      <x:c r="I64" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J64" s="0">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="K64" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L64" s="4">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="M64" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N64" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="24" customHeight="1">
+      <x:c r="A65" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B65" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C65" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Cli_8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D65" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E65" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F65" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G65" s="4">
+        <x:v>10601</x:v>
+      </x:c>
+      <x:c r="H65" s="6">
+        <x:v>36.83</x:v>
+      </x:c>
+      <x:c r="I65" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J65" s="0">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="K65" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L65" s="4">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="M65" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N65" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="24" customHeight="1">
+      <x:c r="A66" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B66" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C66" s="1" t="inlineStr">
+        <x:is>
           <x:t>Cli_9</x:t>
         </x:is>
       </x:c>
-      <x:c r="D53" s="1" t="inlineStr">
+      <x:c r="D66" s="1" t="inlineStr">
         <x:is>
           <x:t>INCONCLUSIVE</x:t>
         </x:is>
       </x:c>
-      <x:c r="E53" s="5">
-        <x:v>0.0</x:v>
-      </x:c>
-      <x:c r="F53" s="4">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G53" s="4">
+      <x:c r="E66" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+      <x:c r="F66" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G66" s="4">
         <x:v>12531</x:v>
       </x:c>
-      <x:c r="H53" s="6">
+      <x:c r="H66" s="6">
         <x:v>50.14</x:v>
       </x:c>
-      <x:c r="I53" s="16">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J53" s="0">
+      <x:c r="I66" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J66" s="0">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="K53" s="4">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L53" s="4">
+      <x:c r="K66" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L66" s="4">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="M53" s="4">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N53" s="5">
-        <x:v>0.0</x:v>
-      </x:c>
+      <x:c r="M66" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N66" s="5">
+        <x:v>0.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="24" customHeight="1">
+      <x:c r="A67" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B67" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C67" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D67" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E67" s="5"/>
+      <x:c r="F67" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G67" s="4">
+        <x:v>10591</x:v>
+      </x:c>
+      <x:c r="H67" s="6">
+        <x:v>26.88</x:v>
+      </x:c>
+      <x:c r="I67" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J67" s="0"/>
+      <x:c r="K67" s="4"/>
+      <x:c r="L67" s="4"/>
+      <x:c r="M67" s="4"/>
+      <x:c r="N67" s="5"/>
+    </x:row>
+    <x:row r="68" ht="24" customHeight="1">
+      <x:c r="A68" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B68" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C68" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D68" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E68" s="5"/>
+      <x:c r="F68" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G68" s="4">
+        <x:v>35664</x:v>
+      </x:c>
+      <x:c r="H68" s="6">
+        <x:v>84.09</x:v>
+      </x:c>
+      <x:c r="I68" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J68" s="0"/>
+      <x:c r="K68" s="4"/>
+      <x:c r="L68" s="4"/>
+      <x:c r="M68" s="4"/>
+      <x:c r="N68" s="5"/>
+    </x:row>
+    <x:row r="69" ht="24" customHeight="1">
+      <x:c r="A69" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B69" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C69" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_11</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D69" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E69" s="5">
+        <x:v>0.5964</x:v>
+      </x:c>
+      <x:c r="F69" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G69" s="4">
+        <x:v>26544</x:v>
+      </x:c>
+      <x:c r="H69" s="6">
+        <x:v>67.5</x:v>
+      </x:c>
+      <x:c r="I69" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J69" s="0">
+        <x:v>778</x:v>
+      </x:c>
+      <x:c r="K69" s="4">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="L69" s="4">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="M69" s="4">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="N69" s="5">
+        <x:v>0.3151</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="24" customHeight="1">
+      <x:c r="A70" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B70" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C70" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_12</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D70" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E70" s="5">
+        <x:v>0.9773000000000001</x:v>
+      </x:c>
+      <x:c r="F70" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G70" s="4">
+        <x:v>13861</x:v>
+      </x:c>
+      <x:c r="H70" s="6">
+        <x:v>58.22</x:v>
+      </x:c>
+      <x:c r="I70" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J70" s="0">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="K70" s="4">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="L70" s="4">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="M70" s="4">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="N70" s="5">
+        <x:v>0.7917000000000001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="24" customHeight="1">
+      <x:c r="A71" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B71" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C71" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D71" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E71" s="5"/>
+      <x:c r="F71" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G71" s="4"/>
+      <x:c r="H71" s="6"/>
+      <x:c r="I71" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J71" s="0"/>
+      <x:c r="K71" s="4"/>
+      <x:c r="L71" s="4"/>
+      <x:c r="M71" s="4"/>
+      <x:c r="N71" s="5"/>
+    </x:row>
+    <x:row r="72" ht="24" customHeight="1">
+      <x:c r="A72" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B72" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C72" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D72" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E72" s="5"/>
+      <x:c r="F72" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G72" s="4"/>
+      <x:c r="H72" s="6"/>
+      <x:c r="I72" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J72" s="0"/>
+      <x:c r="K72" s="4"/>
+      <x:c r="L72" s="4"/>
+      <x:c r="M72" s="4"/>
+      <x:c r="N72" s="5"/>
+    </x:row>
+    <x:row r="73" ht="24" customHeight="1">
+      <x:c r="A73" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B73" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C73" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D73" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E73" s="5"/>
+      <x:c r="F73" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G73" s="4"/>
+      <x:c r="H73" s="6"/>
+      <x:c r="I73" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J73" s="0"/>
+      <x:c r="K73" s="4"/>
+      <x:c r="L73" s="4"/>
+      <x:c r="M73" s="4"/>
+      <x:c r="N73" s="5"/>
+    </x:row>
+    <x:row r="74" ht="24" customHeight="1">
+      <x:c r="A74" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B74" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C74" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D74" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E74" s="5"/>
+      <x:c r="F74" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G74" s="4"/>
+      <x:c r="H74" s="6"/>
+      <x:c r="I74" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J74" s="0"/>
+      <x:c r="K74" s="4"/>
+      <x:c r="L74" s="4"/>
+      <x:c r="M74" s="4"/>
+      <x:c r="N74" s="5"/>
+    </x:row>
+    <x:row r="75" ht="24" customHeight="1">
+      <x:c r="A75" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B75" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C75" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D75" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E75" s="5"/>
+      <x:c r="F75" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G75" s="4"/>
+      <x:c r="H75" s="6"/>
+      <x:c r="I75" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J75" s="0"/>
+      <x:c r="K75" s="4"/>
+      <x:c r="L75" s="4"/>
+      <x:c r="M75" s="4"/>
+      <x:c r="N75" s="5"/>
+    </x:row>
+    <x:row r="76" ht="24" customHeight="1">
+      <x:c r="A76" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B76" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C76" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D76" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E76" s="5"/>
+      <x:c r="F76" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G76" s="4"/>
+      <x:c r="H76" s="6"/>
+      <x:c r="I76" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J76" s="0"/>
+      <x:c r="K76" s="4"/>
+      <x:c r="L76" s="4"/>
+      <x:c r="M76" s="4"/>
+      <x:c r="N76" s="5"/>
+    </x:row>
+    <x:row r="77" ht="24" customHeight="1">
+      <x:c r="A77" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B77" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C77" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D77" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E77" s="5">
+        <x:v>0.8452</x:v>
+      </x:c>
+      <x:c r="F77" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G77" s="4"/>
+      <x:c r="H77" s="6"/>
+      <x:c r="I77" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J77" s="0">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="K77" s="4">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="L77" s="4">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="M77" s="4">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="N77" s="5">
+        <x:v>0.7115</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="24" customHeight="1">
+      <x:c r="A78" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B78" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C78" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D78" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E78" s="5"/>
+      <x:c r="F78" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G78" s="4"/>
+      <x:c r="H78" s="6"/>
+      <x:c r="I78" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J78" s="0"/>
+      <x:c r="K78" s="4"/>
+      <x:c r="L78" s="4"/>
+      <x:c r="M78" s="4"/>
+      <x:c r="N78" s="5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Gemini: add test results for Closure (13-32, count: 20)
</commit_message>
<xml_diff>
--- a/Gemini-3.8-flash/summary.xlsx
+++ b/Gemini-3.8-flash/summary.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N98" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="row_type"/>
     <x:tableColumn id="2" name="round"/>
@@ -412,16 +412,16 @@
         <x:v>Results</x:v>
       </x:c>
       <x:c r="C6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$78,"Round1")</x:f>
-        <x:v>77</x:v>
+        <x:f>COUNTIF(Data!$B$2:$B$98,"Round1")</x:f>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$78,"Round2")</x:f>
+        <x:f>COUNTIF(Data!$B$2:$B$98,"Round2")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="11">
-        <x:f>COUNTA(Data!$C$2:$C$78)</x:f>
-        <x:v>77</x:v>
+        <x:f>COUNTA(Data!$C$2:$C$98)</x:f>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -435,16 +435,16 @@
         <x:v>Average line coverage</x:v>
       </x:c>
       <x:c r="C7" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$E$2:$E$78,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$78,"Round1",Data!$E$2:$E$78))</x:f>
-        <x:v>0.3495192307692308</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$E$2:$E$98,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$98,"Round1",Data!$E$2:$E$98))</x:f>
+        <x:v>0.35690925925925926</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$E$2:$E$78,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$78,"Round2",Data!$E$2:$E$78))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$E$2:$E$98,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$98,"Round2",Data!$E$2:$E$98))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E7" s="12">
-        <x:f>IF(COUNT(Data!$E$2:$E$78)=0,"",AVERAGE(Data!$E$2:$E$78))</x:f>
-        <x:v>0.3495192307692308</x:v>
+        <x:f>IF(COUNT(Data!$E$2:$E$98)=0,"",AVERAGE(Data!$E$2:$E$98))</x:f>
+        <x:v>0.35690925925925926</x:v>
       </x:c>
       <x:c r="F7" s="1"/>
       <x:c r="G7" s="1"/>
@@ -460,16 +460,16 @@
         </x:is>
       </x:c>
       <x:c r="C8" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$N$2:$N$78,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$78,"Round1",Data!$N$2:$N$78))</x:f>
-        <x:v>0.2913882352941176</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$N$2:$N$98,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$98,"Round1",Data!$N$2:$N$98))</x:f>
+        <x:v>0.30040754716981133</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$N$2:$N$78,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$78,"Round2",Data!$N$2:$N$78))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$N$2:$N$98,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$98,"Round2",Data!$N$2:$N$98))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E8" s="12">
-        <x:f>IF(COUNT(Data!$N$2:$N$78)=0,"",AVERAGE(Data!$N$2:$N$78))</x:f>
-        <x:v>0.2913882352941176</x:v>
+        <x:f>IF(COUNT(Data!$N$2:$N$98)=0,"",AVERAGE(Data!$N$2:$N$98))</x:f>
+        <x:v>0.30040754716981133</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -483,15 +483,15 @@
         <x:v>Revealing results</x:v>
       </x:c>
       <x:c r="C9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$78,"Round1",Data!$F$2:$F$78)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$98,"Round1",Data!$F$2:$F$98)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$78,"Round2",Data!$F$2:$F$78)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$98,"Round2",Data!$F$2:$F$98)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="11">
-        <x:f>SUM(Data!$F$2:$F$78)</x:f>
+        <x:f>SUM(Data!$F$2:$F$98)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="1"/>
@@ -529,16 +529,16 @@
         <x:v>Total tokens</x:v>
       </x:c>
       <x:c r="C11" s="10">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$G$2:$G$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$G$2:$G$78))</x:f>
-        <x:v>821823</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$G$2:$G$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$G$2:$G$98))</x:f>
+        <x:v>837908</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$G$2:$G$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$G$2:$G$78))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$G$2:$G$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$G$2:$G$98))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E11" s="11">
-        <x:f>IF(COUNT(Data!$G$2:$G$78)=0,"",SUM(Data!$G$2:$G$78))</x:f>
-        <x:v>821823</x:v>
+        <x:f>IF(COUNT(Data!$G$2:$G$98)=0,"",SUM(Data!$G$2:$G$98))</x:f>
+        <x:v>837908</x:v>
       </x:c>
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
@@ -552,16 +552,16 @@
         <x:v>Generation time (seconds)</x:v>
       </x:c>
       <x:c r="C12" s="6">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$H$2:$H$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$H$2:$H$78))</x:f>
-        <x:v>3210.91</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$H$2:$H$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$H$2:$H$98))</x:f>
+        <x:v>3309.59</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$H$2:$H$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$H$2:$H$78))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$H$2:$H$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$H$2:$H$98))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E12" s="13">
-        <x:f>IF(COUNT(Data!$H$2:$H$78)=0,"",SUM(Data!$H$2:$H$78))</x:f>
-        <x:v>3210.91</x:v>
+        <x:f>IF(COUNT(Data!$H$2:$H$98)=0,"",SUM(Data!$H$2:$H$98))</x:f>
+        <x:v>3309.59</x:v>
       </x:c>
       <x:c r="F12" s="1"/>
       <x:c r="G12" s="1"/>
@@ -575,16 +575,16 @@
         <x:v>Coverage records</x:v>
       </x:c>
       <x:c r="C13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$E$2:$E$78,"&lt;&gt;")</x:f>
-        <x:v>52</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$E$2:$E$98,"&lt;&gt;")</x:f>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="D13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$E$2:$E$78,"&lt;&gt;")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$E$2:$E$98,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="14">
-        <x:f>COUNT(Data!$E$2:$E$78)</x:f>
-        <x:v>52</x:v>
+        <x:f>COUNT(Data!$E$2:$E$98)</x:f>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="F13" s="1"/>
       <x:c r="G13" s="1"/>
@@ -600,16 +600,16 @@
         </x:is>
       </x:c>
       <x:c r="C14" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$J$2:$J$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$J$2:$J$78))</x:f>
-        <x:v>11941</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$J$2:$J$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$J$2:$J$98))</x:f>
+        <x:v>12721</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$J$2:$J$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$J$2:$J$78))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$J$2:$J$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$J$2:$J$98))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E14" s="4">
-        <x:f>IF(COUNT(Data!$J$2:$J$78)=0,"",SUM(Data!$J$2:$J$78))</x:f>
-        <x:v>11941</x:v>
+        <x:f>IF(COUNT(Data!$J$2:$J$98)=0,"",SUM(Data!$J$2:$J$98))</x:f>
+        <x:v>12721</x:v>
       </x:c>
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
@@ -625,16 +625,16 @@
         </x:is>
       </x:c>
       <x:c r="C15" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$K$2:$K$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$K$2:$K$78))</x:f>
-        <x:v>5813</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$K$2:$K$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$K$2:$K$98))</x:f>
+        <x:v>5913</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$K$2:$K$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$K$2:$K$78))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$K$2:$K$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$K$2:$K$98))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E15" s="4">
-        <x:f>IF(COUNT(Data!$K$2:$K$78)=0,"",SUM(Data!$K$2:$K$78))</x:f>
-        <x:v>5813</x:v>
+        <x:f>IF(COUNT(Data!$K$2:$K$98)=0,"",SUM(Data!$K$2:$K$98))</x:f>
+        <x:v>5913</x:v>
       </x:c>
       <x:c r="F15" s="1"/>
       <x:c r="G15" s="1"/>
@@ -650,16 +650,16 @@
         </x:is>
       </x:c>
       <x:c r="C16" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$L$2:$L$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$L$2:$L$78))</x:f>
-        <x:v>6480</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$L$2:$L$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$L$2:$L$98))</x:f>
+        <x:v>7008</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$L$2:$L$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$L$2:$L$78))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$L$2:$L$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$L$2:$L$98))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E16" s="4">
-        <x:f>IF(COUNT(Data!$L$2:$L$78)=0,"",SUM(Data!$L$2:$L$78))</x:f>
-        <x:v>6480</x:v>
+        <x:f>IF(COUNT(Data!$L$2:$L$98)=0,"",SUM(Data!$L$2:$L$98))</x:f>
+        <x:v>7008</x:v>
       </x:c>
       <x:c r="F16" s="1"/>
       <x:c r="G16" s="1"/>
@@ -675,16 +675,16 @@
         </x:is>
       </x:c>
       <x:c r="C17" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$M$2:$M$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round1",Data!$M$2:$M$78))</x:f>
-        <x:v>2409</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$M$2:$M$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$M$2:$M$98))</x:f>
+        <x:v>2443</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$M$2:$M$78,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$78,"Round2",Data!$M$2:$M$78))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$M$2:$M$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$M$2:$M$98))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E17" s="4">
-        <x:f>IF(COUNT(Data!$M$2:$M$78)=0,"",SUM(Data!$M$2:$M$78))</x:f>
-        <x:v>2409</x:v>
+        <x:f>IF(COUNT(Data!$M$2:$M$98)=0,"",SUM(Data!$M$2:$M$98))</x:f>
+        <x:v>2443</x:v>
       </x:c>
       <x:c r="F17" s="1"/>
       <x:c r="G17" s="1"/>
@@ -718,15 +718,15 @@
         <x:v>REVEALING</x:v>
       </x:c>
       <x:c r="C19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$D$2:$D$78,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$D$2:$D$98,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$D$2:$D$78,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$D$2:$D$98,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$78,"REVEALING")</x:f>
+        <x:f>COUNTIF(Data!$D$2:$D$98,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="1"/>
@@ -741,16 +741,16 @@
         <x:v>NOT_REVEALING</x:v>
       </x:c>
       <x:c r="C20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$D$2:$D$78,"NOT_REVEALING")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$D$2:$D$98,"NOT_REVEALING")</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$D$2:$D$78,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$D$2:$D$98,"NOT_REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E20" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$78,"NOT_REVEALING")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$98,"NOT_REVEALING")</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="F20" s="1"/>
       <x:c r="G20" s="1"/>
@@ -764,16 +764,16 @@
         <x:v>NOT_AVAILABLE</x:v>
       </x:c>
       <x:c r="C21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$D$2:$D$78,"NOT_AVAILABLE")</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$D$2:$D$98,"NOT_AVAILABLE")</x:f>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$D$2:$D$78,"NOT_AVAILABLE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$D$2:$D$98,"NOT_AVAILABLE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$78,"NOT_AVAILABLE")</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$98,"NOT_AVAILABLE")</x:f>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="F21" s="1"/>
       <x:c r="G21" s="1"/>
@@ -787,16 +787,16 @@
         <x:v>INCONCLUSIVE</x:v>
       </x:c>
       <x:c r="C22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round1",Data!$D$2:$D$78,"INCONCLUSIVE")</x:f>
-        <x:v>38</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$D$2:$D$98,"INCONCLUSIVE")</x:f>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$78,"Round2",Data!$D$2:$D$78,"INCONCLUSIVE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$D$2:$D$98,"INCONCLUSIVE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$78,"INCONCLUSIVE")</x:f>
-        <x:v>38</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$98,"INCONCLUSIVE")</x:f>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F22" s="1"/>
       <x:c r="G22" s="1"/>
@@ -836,7 +836,7 @@
       <x:c r="A25" s="1"/>
       <x:c r="B25" s="3" t="inlineStr">
         <x:is>
-          <x:t>Updated: 2026-09-30 05:32:32 +0700</x:t>
+          <x:t>Updated: 2026-09-30 05:39:44 +0700</x:t>
         </x:is>
       </x:c>
       <x:c r="C25" s="3"/>
@@ -4330,7 +4330,7 @@
       </x:c>
       <x:c r="C71" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_2</x:t>
+          <x:t>Closure_13</x:t>
         </x:is>
       </x:c>
       <x:c r="D71" s="1" t="inlineStr">
@@ -4342,8 +4342,12 @@
       <x:c r="F71" s="4">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G71" s="4"/>
-      <x:c r="H71" s="6"/>
+      <x:c r="G71" s="4">
+        <x:v>8950</x:v>
+      </x:c>
+      <x:c r="H71" s="6">
+        <x:v>45.61</x:v>
+      </x:c>
       <x:c r="I71" s="16">
         <x:v>1</x:v>
       </x:c>
@@ -4366,7 +4370,7 @@
       </x:c>
       <x:c r="C72" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_3</x:t>
+          <x:t>Closure_14</x:t>
         </x:is>
       </x:c>
       <x:c r="D72" s="1" t="inlineStr">
@@ -4402,7 +4406,7 @@
       </x:c>
       <x:c r="C73" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_4</x:t>
+          <x:t>Closure_15</x:t>
         </x:is>
       </x:c>
       <x:c r="D73" s="1" t="inlineStr">
@@ -4438,7 +4442,7 @@
       </x:c>
       <x:c r="C74" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_5</x:t>
+          <x:t>Closure_16</x:t>
         </x:is>
       </x:c>
       <x:c r="D74" s="1" t="inlineStr">
@@ -4474,7 +4478,7 @@
       </x:c>
       <x:c r="C75" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_6</x:t>
+          <x:t>Closure_17</x:t>
         </x:is>
       </x:c>
       <x:c r="D75" s="1" t="inlineStr">
@@ -4510,7 +4514,7 @@
       </x:c>
       <x:c r="C76" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_7</x:t>
+          <x:t>Closure_18</x:t>
         </x:is>
       </x:c>
       <x:c r="D76" s="1" t="inlineStr">
@@ -4546,17 +4550,15 @@
       </x:c>
       <x:c r="C77" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_8</x:t>
+          <x:t>Closure_19</x:t>
         </x:is>
       </x:c>
       <x:c r="D77" s="1" t="inlineStr">
         <x:is>
-          <x:t>INCONCLUSIVE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E77" s="5">
-        <x:v>0.8452</x:v>
-      </x:c>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E77" s="5"/>
       <x:c r="F77" s="4">
         <x:v>0</x:v>
       </x:c>
@@ -4565,21 +4567,11 @@
       <x:c r="I77" s="16">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J77" s="0">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="K77" s="4">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="L77" s="4">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="M77" s="4">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="N77" s="5">
-        <x:v>0.7115</x:v>
-      </x:c>
+      <x:c r="J77" s="0"/>
+      <x:c r="K77" s="4"/>
+      <x:c r="L77" s="4"/>
+      <x:c r="M77" s="4"/>
+      <x:c r="N77" s="5"/>
     </x:row>
     <x:row r="78" ht="24" customHeight="1">
       <x:c r="A78" s="1" t="inlineStr">
@@ -4594,7 +4586,7 @@
       </x:c>
       <x:c r="C78" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_9</x:t>
+          <x:t>Closure_2</x:t>
         </x:is>
       </x:c>
       <x:c r="D78" s="1" t="inlineStr">
@@ -4616,6 +4608,766 @@
       <x:c r="L78" s="4"/>
       <x:c r="M78" s="4"/>
       <x:c r="N78" s="5"/>
+    </x:row>
+    <x:row r="79" ht="24" customHeight="1">
+      <x:c r="A79" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B79" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C79" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D79" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E79" s="5">
+        <x:v>0.0981</x:v>
+      </x:c>
+      <x:c r="F79" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G79" s="4"/>
+      <x:c r="H79" s="6"/>
+      <x:c r="I79" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J79" s="0">
+        <x:v>754</x:v>
+      </x:c>
+      <x:c r="K79" s="4">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="L79" s="4">
+        <x:v>526</x:v>
+      </x:c>
+      <x:c r="M79" s="4">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="N79" s="5">
+        <x:v>0.0608</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="24" customHeight="1">
+      <x:c r="A80" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B80" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C80" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_21</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D80" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E80" s="5"/>
+      <x:c r="F80" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G80" s="4"/>
+      <x:c r="H80" s="6"/>
+      <x:c r="I80" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J80" s="0"/>
+      <x:c r="K80" s="4"/>
+      <x:c r="L80" s="4"/>
+      <x:c r="M80" s="4"/>
+      <x:c r="N80" s="5"/>
+    </x:row>
+    <x:row r="81" ht="24" customHeight="1">
+      <x:c r="A81" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B81" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C81" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D81" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E81" s="5"/>
+      <x:c r="F81" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G81" s="4"/>
+      <x:c r="H81" s="6"/>
+      <x:c r="I81" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J81" s="0"/>
+      <x:c r="K81" s="4"/>
+      <x:c r="L81" s="4"/>
+      <x:c r="M81" s="4"/>
+      <x:c r="N81" s="5"/>
+    </x:row>
+    <x:row r="82" ht="24" customHeight="1">
+      <x:c r="A82" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B82" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C82" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_23</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D82" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E82" s="5"/>
+      <x:c r="F82" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G82" s="4"/>
+      <x:c r="H82" s="6"/>
+      <x:c r="I82" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J82" s="0"/>
+      <x:c r="K82" s="4"/>
+      <x:c r="L82" s="4"/>
+      <x:c r="M82" s="4"/>
+      <x:c r="N82" s="5"/>
+    </x:row>
+    <x:row r="83" ht="24" customHeight="1">
+      <x:c r="A83" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B83" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C83" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_24</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D83" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E83" s="5"/>
+      <x:c r="F83" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G83" s="4"/>
+      <x:c r="H83" s="6"/>
+      <x:c r="I83" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J83" s="0"/>
+      <x:c r="K83" s="4"/>
+      <x:c r="L83" s="4"/>
+      <x:c r="M83" s="4"/>
+      <x:c r="N83" s="5"/>
+    </x:row>
+    <x:row r="84" ht="24" customHeight="1">
+      <x:c r="A84" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B84" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C84" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_25</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D84" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E84" s="5"/>
+      <x:c r="F84" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G84" s="4"/>
+      <x:c r="H84" s="6"/>
+      <x:c r="I84" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J84" s="0"/>
+      <x:c r="K84" s="4"/>
+      <x:c r="L84" s="4"/>
+      <x:c r="M84" s="4"/>
+      <x:c r="N84" s="5"/>
+    </x:row>
+    <x:row r="85" ht="24" customHeight="1">
+      <x:c r="A85" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B85" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C85" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_26</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D85" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E85" s="5"/>
+      <x:c r="F85" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G85" s="4"/>
+      <x:c r="H85" s="6"/>
+      <x:c r="I85" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J85" s="0"/>
+      <x:c r="K85" s="4"/>
+      <x:c r="L85" s="4"/>
+      <x:c r="M85" s="4"/>
+      <x:c r="N85" s="5"/>
+    </x:row>
+    <x:row r="86" ht="24" customHeight="1">
+      <x:c r="A86" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B86" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C86" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_27</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D86" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E86" s="5"/>
+      <x:c r="F86" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G86" s="4"/>
+      <x:c r="H86" s="6"/>
+      <x:c r="I86" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J86" s="0"/>
+      <x:c r="K86" s="4"/>
+      <x:c r="L86" s="4"/>
+      <x:c r="M86" s="4"/>
+      <x:c r="N86" s="5"/>
+    </x:row>
+    <x:row r="87" ht="24" customHeight="1">
+      <x:c r="A87" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B87" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C87" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_28</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D87" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_REVEALING</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E87" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="F87" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G87" s="4">
+        <x:v>7135</x:v>
+      </x:c>
+      <x:c r="H87" s="6">
+        <x:v>53.07</x:v>
+      </x:c>
+      <x:c r="I87" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J87" s="0">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="K87" s="4">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="L87" s="4">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="M87" s="4">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="N87" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="24" customHeight="1">
+      <x:c r="A88" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B88" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C88" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_29</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D88" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E88" s="5"/>
+      <x:c r="F88" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G88" s="4"/>
+      <x:c r="H88" s="6"/>
+      <x:c r="I88" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J88" s="0"/>
+      <x:c r="K88" s="4"/>
+      <x:c r="L88" s="4"/>
+      <x:c r="M88" s="4"/>
+      <x:c r="N88" s="5"/>
+    </x:row>
+    <x:row r="89" ht="24" customHeight="1">
+      <x:c r="A89" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B89" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C89" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D89" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E89" s="5"/>
+      <x:c r="F89" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G89" s="4"/>
+      <x:c r="H89" s="6"/>
+      <x:c r="I89" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J89" s="0"/>
+      <x:c r="K89" s="4"/>
+      <x:c r="L89" s="4"/>
+      <x:c r="M89" s="4"/>
+      <x:c r="N89" s="5"/>
+    </x:row>
+    <x:row r="90" ht="24" customHeight="1">
+      <x:c r="A90" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B90" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C90" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_30</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D90" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E90" s="5"/>
+      <x:c r="F90" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G90" s="4"/>
+      <x:c r="H90" s="6"/>
+      <x:c r="I90" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J90" s="0"/>
+      <x:c r="K90" s="4"/>
+      <x:c r="L90" s="4"/>
+      <x:c r="M90" s="4"/>
+      <x:c r="N90" s="5"/>
+    </x:row>
+    <x:row r="91" ht="24" customHeight="1">
+      <x:c r="A91" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B91" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C91" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_31</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D91" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E91" s="5"/>
+      <x:c r="F91" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G91" s="4"/>
+      <x:c r="H91" s="6"/>
+      <x:c r="I91" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J91" s="0"/>
+      <x:c r="K91" s="4"/>
+      <x:c r="L91" s="4"/>
+      <x:c r="M91" s="4"/>
+      <x:c r="N91" s="5"/>
+    </x:row>
+    <x:row r="92" ht="24" customHeight="1">
+      <x:c r="A92" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B92" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C92" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_32</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D92" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E92" s="5"/>
+      <x:c r="F92" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G92" s="4"/>
+      <x:c r="H92" s="6"/>
+      <x:c r="I92" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J92" s="0"/>
+      <x:c r="K92" s="4"/>
+      <x:c r="L92" s="4"/>
+      <x:c r="M92" s="4"/>
+      <x:c r="N92" s="5"/>
+    </x:row>
+    <x:row r="93" ht="24" customHeight="1">
+      <x:c r="A93" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B93" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C93" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D93" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E93" s="5"/>
+      <x:c r="F93" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G93" s="4"/>
+      <x:c r="H93" s="6"/>
+      <x:c r="I93" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J93" s="0"/>
+      <x:c r="K93" s="4"/>
+      <x:c r="L93" s="4"/>
+      <x:c r="M93" s="4"/>
+      <x:c r="N93" s="5"/>
+    </x:row>
+    <x:row r="94" ht="24" customHeight="1">
+      <x:c r="A94" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B94" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C94" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D94" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E94" s="5"/>
+      <x:c r="F94" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G94" s="4"/>
+      <x:c r="H94" s="6"/>
+      <x:c r="I94" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J94" s="0"/>
+      <x:c r="K94" s="4"/>
+      <x:c r="L94" s="4"/>
+      <x:c r="M94" s="4"/>
+      <x:c r="N94" s="5"/>
+    </x:row>
+    <x:row r="95" ht="24" customHeight="1">
+      <x:c r="A95" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B95" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C95" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D95" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E95" s="5"/>
+      <x:c r="F95" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G95" s="4"/>
+      <x:c r="H95" s="6"/>
+      <x:c r="I95" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J95" s="0"/>
+      <x:c r="K95" s="4"/>
+      <x:c r="L95" s="4"/>
+      <x:c r="M95" s="4"/>
+      <x:c r="N95" s="5"/>
+    </x:row>
+    <x:row r="96" ht="24" customHeight="1">
+      <x:c r="A96" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B96" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C96" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D96" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E96" s="5"/>
+      <x:c r="F96" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G96" s="4"/>
+      <x:c r="H96" s="6"/>
+      <x:c r="I96" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J96" s="0"/>
+      <x:c r="K96" s="4"/>
+      <x:c r="L96" s="4"/>
+      <x:c r="M96" s="4"/>
+      <x:c r="N96" s="5"/>
+    </x:row>
+    <x:row r="97" ht="24" customHeight="1">
+      <x:c r="A97" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B97" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C97" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D97" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E97" s="5">
+        <x:v>0.8452</x:v>
+      </x:c>
+      <x:c r="F97" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G97" s="4"/>
+      <x:c r="H97" s="6"/>
+      <x:c r="I97" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J97" s="0">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="K97" s="4">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="L97" s="4">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="M97" s="4">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="N97" s="5">
+        <x:v>0.7115</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="24" customHeight="1">
+      <x:c r="A98" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B98" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C98" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D98" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E98" s="5"/>
+      <x:c r="F98" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G98" s="4"/>
+      <x:c r="H98" s="6"/>
+      <x:c r="I98" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J98" s="0"/>
+      <x:c r="K98" s="4"/>
+      <x:c r="L98" s="4"/>
+      <x:c r="M98" s="4"/>
+      <x:c r="N98" s="5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Gemini: add test results for Closure (33-55, count: 22)
</commit_message>
<xml_diff>
--- a/Gemini-3.8-flash/summary.xlsx
+++ b/Gemini-3.8-flash/summary.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N98" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N120" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="row_type"/>
     <x:tableColumn id="2" name="round"/>
@@ -412,16 +412,16 @@
         <x:v>Results</x:v>
       </x:c>
       <x:c r="C6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$98,"Round1")</x:f>
-        <x:v>97</x:v>
+        <x:f>COUNTIF(Data!$B$2:$B$120,"Round1")</x:f>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="D6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$98,"Round2")</x:f>
+        <x:f>COUNTIF(Data!$B$2:$B$120,"Round2")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="11">
-        <x:f>COUNTA(Data!$C$2:$C$98)</x:f>
-        <x:v>97</x:v>
+        <x:f>COUNTA(Data!$C$2:$C$120)</x:f>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -435,16 +435,16 @@
         <x:v>Average line coverage</x:v>
       </x:c>
       <x:c r="C7" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$E$2:$E$98,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$98,"Round1",Data!$E$2:$E$98))</x:f>
-        <x:v>0.35690925925925926</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$E$2:$E$120,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$120,"Round1",Data!$E$2:$E$120))</x:f>
+        <x:v>0.37134821428571435</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$E$2:$E$98,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$98,"Round2",Data!$E$2:$E$98))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$E$2:$E$120,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$120,"Round2",Data!$E$2:$E$120))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E7" s="12">
-        <x:f>IF(COUNT(Data!$E$2:$E$98)=0,"",AVERAGE(Data!$E$2:$E$98))</x:f>
-        <x:v>0.35690925925925926</x:v>
+        <x:f>IF(COUNT(Data!$E$2:$E$120)=0,"",AVERAGE(Data!$E$2:$E$120))</x:f>
+        <x:v>0.37134821428571435</x:v>
       </x:c>
       <x:c r="F7" s="1"/>
       <x:c r="G7" s="1"/>
@@ -460,16 +460,16 @@
         </x:is>
       </x:c>
       <x:c r="C8" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$N$2:$N$98,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$98,"Round1",Data!$N$2:$N$98))</x:f>
-        <x:v>0.30040754716981133</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$N$2:$N$120,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$120,"Round1",Data!$N$2:$N$120))</x:f>
+        <x:v>0.31776</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$N$2:$N$98,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$98,"Round2",Data!$N$2:$N$98))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$N$2:$N$120,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$120,"Round2",Data!$N$2:$N$120))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E8" s="12">
-        <x:f>IF(COUNT(Data!$N$2:$N$98)=0,"",AVERAGE(Data!$N$2:$N$98))</x:f>
-        <x:v>0.30040754716981133</x:v>
+        <x:f>IF(COUNT(Data!$N$2:$N$120)=0,"",AVERAGE(Data!$N$2:$N$120))</x:f>
+        <x:v>0.31776</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -483,15 +483,15 @@
         <x:v>Revealing results</x:v>
       </x:c>
       <x:c r="C9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$98,"Round1",Data!$F$2:$F$98)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$120,"Round1",Data!$F$2:$F$120)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$98,"Round2",Data!$F$2:$F$98)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$120,"Round2",Data!$F$2:$F$120)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="11">
-        <x:f>SUM(Data!$F$2:$F$98)</x:f>
+        <x:f>SUM(Data!$F$2:$F$120)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="1"/>
@@ -529,16 +529,16 @@
         <x:v>Total tokens</x:v>
       </x:c>
       <x:c r="C11" s="10">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$G$2:$G$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$G$2:$G$98))</x:f>
-        <x:v>837908</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$G$2:$G$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$G$2:$G$120))</x:f>
+        <x:v>861110</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$G$2:$G$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$G$2:$G$98))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$G$2:$G$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$G$2:$G$120))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E11" s="11">
-        <x:f>IF(COUNT(Data!$G$2:$G$98)=0,"",SUM(Data!$G$2:$G$98))</x:f>
-        <x:v>837908</x:v>
+        <x:f>IF(COUNT(Data!$G$2:$G$120)=0,"",SUM(Data!$G$2:$G$120))</x:f>
+        <x:v>861110</x:v>
       </x:c>
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
@@ -552,16 +552,16 @@
         <x:v>Generation time (seconds)</x:v>
       </x:c>
       <x:c r="C12" s="6">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$H$2:$H$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$H$2:$H$98))</x:f>
-        <x:v>3309.59</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$H$2:$H$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$H$2:$H$120))</x:f>
+        <x:v>3425.85</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$H$2:$H$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$H$2:$H$98))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$H$2:$H$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$H$2:$H$120))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E12" s="13">
-        <x:f>IF(COUNT(Data!$H$2:$H$98)=0,"",SUM(Data!$H$2:$H$98))</x:f>
-        <x:v>3309.59</x:v>
+        <x:f>IF(COUNT(Data!$H$2:$H$120)=0,"",SUM(Data!$H$2:$H$120))</x:f>
+        <x:v>3425.85</x:v>
       </x:c>
       <x:c r="F12" s="1"/>
       <x:c r="G12" s="1"/>
@@ -575,16 +575,16 @@
         <x:v>Coverage records</x:v>
       </x:c>
       <x:c r="C13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$E$2:$E$98,"&lt;&gt;")</x:f>
-        <x:v>54</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$E$2:$E$120,"&lt;&gt;")</x:f>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$E$2:$E$98,"&lt;&gt;")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$E$2:$E$120,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="14">
-        <x:f>COUNT(Data!$E$2:$E$98)</x:f>
-        <x:v>54</x:v>
+        <x:f>COUNT(Data!$E$2:$E$120)</x:f>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="F13" s="1"/>
       <x:c r="G13" s="1"/>
@@ -600,16 +600,16 @@
         </x:is>
       </x:c>
       <x:c r="C14" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$J$2:$J$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$J$2:$J$98))</x:f>
-        <x:v>12721</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$J$2:$J$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$J$2:$J$120))</x:f>
+        <x:v>12942</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$J$2:$J$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$J$2:$J$98))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$J$2:$J$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$J$2:$J$120))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E14" s="4">
-        <x:f>IF(COUNT(Data!$J$2:$J$98)=0,"",SUM(Data!$J$2:$J$98))</x:f>
-        <x:v>12721</x:v>
+        <x:f>IF(COUNT(Data!$J$2:$J$120)=0,"",SUM(Data!$J$2:$J$120))</x:f>
+        <x:v>12942</x:v>
       </x:c>
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
@@ -625,16 +625,16 @@
         </x:is>
       </x:c>
       <x:c r="C15" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$K$2:$K$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$K$2:$K$98))</x:f>
-        <x:v>5913</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$K$2:$K$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$K$2:$K$120))</x:f>
+        <x:v>6081</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$K$2:$K$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$K$2:$K$98))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$K$2:$K$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$K$2:$K$120))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E15" s="4">
-        <x:f>IF(COUNT(Data!$K$2:$K$98)=0,"",SUM(Data!$K$2:$K$98))</x:f>
-        <x:v>5913</x:v>
+        <x:f>IF(COUNT(Data!$K$2:$K$120)=0,"",SUM(Data!$K$2:$K$120))</x:f>
+        <x:v>6081</x:v>
       </x:c>
       <x:c r="F15" s="1"/>
       <x:c r="G15" s="1"/>
@@ -650,16 +650,16 @@
         </x:is>
       </x:c>
       <x:c r="C16" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$L$2:$L$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$L$2:$L$98))</x:f>
-        <x:v>7008</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$L$2:$L$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$L$2:$L$120))</x:f>
+        <x:v>7132</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$L$2:$L$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$L$2:$L$98))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$L$2:$L$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$L$2:$L$120))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E16" s="4">
-        <x:f>IF(COUNT(Data!$L$2:$L$98)=0,"",SUM(Data!$L$2:$L$98))</x:f>
-        <x:v>7008</x:v>
+        <x:f>IF(COUNT(Data!$L$2:$L$120)=0,"",SUM(Data!$L$2:$L$120))</x:f>
+        <x:v>7132</x:v>
       </x:c>
       <x:c r="F16" s="1"/>
       <x:c r="G16" s="1"/>
@@ -675,16 +675,16 @@
         </x:is>
       </x:c>
       <x:c r="C17" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$M$2:$M$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round1",Data!$M$2:$M$98))</x:f>
-        <x:v>2443</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$M$2:$M$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$M$2:$M$120))</x:f>
+        <x:v>2539</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$M$2:$M$98,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$98,"Round2",Data!$M$2:$M$98))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$M$2:$M$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$M$2:$M$120))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E17" s="4">
-        <x:f>IF(COUNT(Data!$M$2:$M$98)=0,"",SUM(Data!$M$2:$M$98))</x:f>
-        <x:v>2443</x:v>
+        <x:f>IF(COUNT(Data!$M$2:$M$120)=0,"",SUM(Data!$M$2:$M$120))</x:f>
+        <x:v>2539</x:v>
       </x:c>
       <x:c r="F17" s="1"/>
       <x:c r="G17" s="1"/>
@@ -718,15 +718,15 @@
         <x:v>REVEALING</x:v>
       </x:c>
       <x:c r="C19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$D$2:$D$98,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$D$2:$D$120,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$D$2:$D$98,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$D$2:$D$120,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$98,"REVEALING")</x:f>
+        <x:f>COUNTIF(Data!$D$2:$D$120,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="1"/>
@@ -741,15 +741,15 @@
         <x:v>NOT_REVEALING</x:v>
       </x:c>
       <x:c r="C20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$D$2:$D$98,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$D$2:$D$120,"NOT_REVEALING")</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="D20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$D$2:$D$98,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$D$2:$D$120,"NOT_REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E20" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$98,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIF(Data!$D$2:$D$120,"NOT_REVEALING")</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="F20" s="1"/>
@@ -764,16 +764,16 @@
         <x:v>NOT_AVAILABLE</x:v>
       </x:c>
       <x:c r="C21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$D$2:$D$98,"NOT_AVAILABLE")</x:f>
-        <x:v>43</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$D$2:$D$120,"NOT_AVAILABLE")</x:f>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$D$2:$D$98,"NOT_AVAILABLE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$D$2:$D$120,"NOT_AVAILABLE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$98,"NOT_AVAILABLE")</x:f>
-        <x:v>43</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$120,"NOT_AVAILABLE")</x:f>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F21" s="1"/>
       <x:c r="G21" s="1"/>
@@ -787,16 +787,16 @@
         <x:v>INCONCLUSIVE</x:v>
       </x:c>
       <x:c r="C22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round1",Data!$D$2:$D$98,"INCONCLUSIVE")</x:f>
-        <x:v>39</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$D$2:$D$120,"INCONCLUSIVE")</x:f>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$98,"Round2",Data!$D$2:$D$98,"INCONCLUSIVE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$D$2:$D$120,"INCONCLUSIVE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$98,"INCONCLUSIVE")</x:f>
-        <x:v>39</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$120,"INCONCLUSIVE")</x:f>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="F22" s="1"/>
       <x:c r="G22" s="1"/>
@@ -836,7 +836,7 @@
       <x:c r="A25" s="1"/>
       <x:c r="B25" s="3" t="inlineStr">
         <x:is>
-          <x:t>Updated: 2026-09-30 05:39:44 +0700</x:t>
+          <x:t>Updated: 2026-09-30 05:45:10 +0700</x:t>
         </x:is>
       </x:c>
       <x:c r="C25" s="3"/>
@@ -5154,7 +5154,7 @@
       </x:c>
       <x:c r="C93" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_4</x:t>
+          <x:t>Closure_33</x:t>
         </x:is>
       </x:c>
       <x:c r="D93" s="1" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </x:c>
       <x:c r="C94" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_5</x:t>
+          <x:t>Closure_34</x:t>
         </x:is>
       </x:c>
       <x:c r="D94" s="1" t="inlineStr">
@@ -5226,7 +5226,7 @@
       </x:c>
       <x:c r="C95" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_6</x:t>
+          <x:t>Closure_35</x:t>
         </x:is>
       </x:c>
       <x:c r="D95" s="1" t="inlineStr">
@@ -5262,7 +5262,7 @@
       </x:c>
       <x:c r="C96" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_7</x:t>
+          <x:t>Closure_36</x:t>
         </x:is>
       </x:c>
       <x:c r="D96" s="1" t="inlineStr">
@@ -5298,17 +5298,15 @@
       </x:c>
       <x:c r="C97" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_8</x:t>
+          <x:t>Closure_37</x:t>
         </x:is>
       </x:c>
       <x:c r="D97" s="1" t="inlineStr">
         <x:is>
-          <x:t>INCONCLUSIVE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E97" s="5">
-        <x:v>0.8452</x:v>
-      </x:c>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E97" s="5"/>
       <x:c r="F97" s="4">
         <x:v>0</x:v>
       </x:c>
@@ -5317,21 +5315,11 @@
       <x:c r="I97" s="16">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J97" s="0">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="K97" s="4">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="L97" s="4">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="M97" s="4">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="N97" s="5">
-        <x:v>0.7115</x:v>
-      </x:c>
+      <x:c r="J97" s="0"/>
+      <x:c r="K97" s="4"/>
+      <x:c r="L97" s="4"/>
+      <x:c r="M97" s="4"/>
+      <x:c r="N97" s="5"/>
     </x:row>
     <x:row r="98" ht="24" customHeight="1">
       <x:c r="A98" s="1" t="inlineStr">
@@ -5346,15 +5334,17 @@
       </x:c>
       <x:c r="C98" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_9</x:t>
+          <x:t>Closure_38</x:t>
         </x:is>
       </x:c>
       <x:c r="D98" s="1" t="inlineStr">
         <x:is>
-          <x:t>NOT_AVAILABLE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E98" s="5"/>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E98" s="5">
+        <x:v>0.6875</x:v>
+      </x:c>
       <x:c r="F98" s="4">
         <x:v>0</x:v>
       </x:c>
@@ -5363,11 +5353,845 @@
       <x:c r="I98" s="16">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J98" s="0"/>
-      <x:c r="K98" s="4"/>
-      <x:c r="L98" s="4"/>
-      <x:c r="M98" s="4"/>
-      <x:c r="N98" s="5"/>
+      <x:c r="J98" s="0">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="K98" s="4">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="L98" s="4">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="M98" s="4">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="N98" s="5">
+        <x:v>0.6718999999999999</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="24" customHeight="1">
+      <x:c r="A99" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B99" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C99" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_39</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D99" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E99" s="5"/>
+      <x:c r="F99" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G99" s="4"/>
+      <x:c r="H99" s="6"/>
+      <x:c r="I99" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J99" s="0"/>
+      <x:c r="K99" s="4"/>
+      <x:c r="L99" s="4"/>
+      <x:c r="M99" s="4"/>
+      <x:c r="N99" s="5"/>
+    </x:row>
+    <x:row r="100" ht="24" customHeight="1">
+      <x:c r="A100" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B100" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C100" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D100" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E100" s="5"/>
+      <x:c r="F100" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G100" s="4"/>
+      <x:c r="H100" s="6"/>
+      <x:c r="I100" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J100" s="0"/>
+      <x:c r="K100" s="4"/>
+      <x:c r="L100" s="4"/>
+      <x:c r="M100" s="4"/>
+      <x:c r="N100" s="5"/>
+    </x:row>
+    <x:row r="101" ht="24" customHeight="1">
+      <x:c r="A101" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B101" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C101" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_40</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D101" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E101" s="5"/>
+      <x:c r="F101" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G101" s="4"/>
+      <x:c r="H101" s="6"/>
+      <x:c r="I101" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J101" s="0"/>
+      <x:c r="K101" s="4"/>
+      <x:c r="L101" s="4"/>
+      <x:c r="M101" s="4"/>
+      <x:c r="N101" s="5"/>
+    </x:row>
+    <x:row r="102" ht="24" customHeight="1">
+      <x:c r="A102" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B102" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C102" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_41</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D102" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E102" s="5"/>
+      <x:c r="F102" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G102" s="4"/>
+      <x:c r="H102" s="6"/>
+      <x:c r="I102" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J102" s="0"/>
+      <x:c r="K102" s="4"/>
+      <x:c r="L102" s="4"/>
+      <x:c r="M102" s="4"/>
+      <x:c r="N102" s="5"/>
+    </x:row>
+    <x:row r="103" ht="24" customHeight="1">
+      <x:c r="A103" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B103" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C103" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_42</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D103" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E103" s="5"/>
+      <x:c r="F103" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G103" s="4"/>
+      <x:c r="H103" s="6"/>
+      <x:c r="I103" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J103" s="0"/>
+      <x:c r="K103" s="4"/>
+      <x:c r="L103" s="4"/>
+      <x:c r="M103" s="4"/>
+      <x:c r="N103" s="5"/>
+    </x:row>
+    <x:row r="104" ht="24" customHeight="1">
+      <x:c r="A104" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B104" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C104" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_43</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D104" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E104" s="5"/>
+      <x:c r="F104" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G104" s="4"/>
+      <x:c r="H104" s="6"/>
+      <x:c r="I104" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J104" s="0"/>
+      <x:c r="K104" s="4"/>
+      <x:c r="L104" s="4"/>
+      <x:c r="M104" s="4"/>
+      <x:c r="N104" s="5"/>
+    </x:row>
+    <x:row r="105" ht="24" customHeight="1">
+      <x:c r="A105" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B105" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C105" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_44</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D105" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E105" s="5">
+        <x:v>0.8349</x:v>
+      </x:c>
+      <x:c r="F105" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G105" s="4"/>
+      <x:c r="H105" s="6"/>
+      <x:c r="I105" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J105" s="0">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="K105" s="4">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="L105" s="4">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="M105" s="4">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="N105" s="5">
+        <x:v>0.8833</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="24" customHeight="1">
+      <x:c r="A106" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B106" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C106" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_45</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D106" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E106" s="5"/>
+      <x:c r="F106" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G106" s="4"/>
+      <x:c r="H106" s="6"/>
+      <x:c r="I106" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J106" s="0"/>
+      <x:c r="K106" s="4"/>
+      <x:c r="L106" s="4"/>
+      <x:c r="M106" s="4"/>
+      <x:c r="N106" s="5"/>
+    </x:row>
+    <x:row r="107" ht="24" customHeight="1">
+      <x:c r="A107" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B107" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C107" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_46</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D107" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E107" s="5"/>
+      <x:c r="F107" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G107" s="4"/>
+      <x:c r="H107" s="6"/>
+      <x:c r="I107" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J107" s="0"/>
+      <x:c r="K107" s="4"/>
+      <x:c r="L107" s="4"/>
+      <x:c r="M107" s="4"/>
+      <x:c r="N107" s="5"/>
+    </x:row>
+    <x:row r="108" ht="24" customHeight="1">
+      <x:c r="A108" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B108" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C108" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_47</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D108" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E108" s="5"/>
+      <x:c r="F108" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G108" s="4">
+        <x:v>16621</x:v>
+      </x:c>
+      <x:c r="H108" s="6">
+        <x:v>96.23</x:v>
+      </x:c>
+      <x:c r="I108" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J108" s="0"/>
+      <x:c r="K108" s="4"/>
+      <x:c r="L108" s="4"/>
+      <x:c r="M108" s="4"/>
+      <x:c r="N108" s="5"/>
+    </x:row>
+    <x:row r="109" ht="24" customHeight="1">
+      <x:c r="A109" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B109" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C109" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_48</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D109" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E109" s="5"/>
+      <x:c r="F109" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G109" s="4"/>
+      <x:c r="H109" s="6"/>
+      <x:c r="I109" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J109" s="0"/>
+      <x:c r="K109" s="4"/>
+      <x:c r="L109" s="4"/>
+      <x:c r="M109" s="4"/>
+      <x:c r="N109" s="5"/>
+    </x:row>
+    <x:row r="110" ht="24" customHeight="1">
+      <x:c r="A110" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B110" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C110" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_49</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D110" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E110" s="5"/>
+      <x:c r="F110" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G110" s="4"/>
+      <x:c r="H110" s="6"/>
+      <x:c r="I110" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J110" s="0"/>
+      <x:c r="K110" s="4"/>
+      <x:c r="L110" s="4"/>
+      <x:c r="M110" s="4"/>
+      <x:c r="N110" s="5"/>
+    </x:row>
+    <x:row r="111" ht="24" customHeight="1">
+      <x:c r="A111" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B111" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C111" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D111" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E111" s="5"/>
+      <x:c r="F111" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G111" s="4"/>
+      <x:c r="H111" s="6"/>
+      <x:c r="I111" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J111" s="0"/>
+      <x:c r="K111" s="4"/>
+      <x:c r="L111" s="4"/>
+      <x:c r="M111" s="4"/>
+      <x:c r="N111" s="5"/>
+    </x:row>
+    <x:row r="112" ht="24" customHeight="1">
+      <x:c r="A112" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B112" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C112" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_50</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D112" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E112" s="5"/>
+      <x:c r="F112" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G112" s="4"/>
+      <x:c r="H112" s="6"/>
+      <x:c r="I112" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J112" s="0"/>
+      <x:c r="K112" s="4"/>
+      <x:c r="L112" s="4"/>
+      <x:c r="M112" s="4"/>
+      <x:c r="N112" s="5"/>
+    </x:row>
+    <x:row r="113" ht="24" customHeight="1">
+      <x:c r="A113" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B113" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C113" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_51</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D113" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E113" s="5"/>
+      <x:c r="F113" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G113" s="4">
+        <x:v>6581</x:v>
+      </x:c>
+      <x:c r="H113" s="6">
+        <x:v>20.03</x:v>
+      </x:c>
+      <x:c r="I113" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J113" s="0"/>
+      <x:c r="K113" s="4"/>
+      <x:c r="L113" s="4"/>
+      <x:c r="M113" s="4"/>
+      <x:c r="N113" s="5"/>
+    </x:row>
+    <x:row r="114" ht="24" customHeight="1">
+      <x:c r="A114" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B114" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C114" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_52</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D114" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E114" s="5"/>
+      <x:c r="F114" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G114" s="4"/>
+      <x:c r="H114" s="6"/>
+      <x:c r="I114" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J114" s="0"/>
+      <x:c r="K114" s="4"/>
+      <x:c r="L114" s="4"/>
+      <x:c r="M114" s="4"/>
+      <x:c r="N114" s="5"/>
+    </x:row>
+    <x:row r="115" ht="24" customHeight="1">
+      <x:c r="A115" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B115" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C115" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_53</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D115" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E115" s="5"/>
+      <x:c r="F115" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G115" s="4"/>
+      <x:c r="H115" s="6"/>
+      <x:c r="I115" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J115" s="0"/>
+      <x:c r="K115" s="4"/>
+      <x:c r="L115" s="4"/>
+      <x:c r="M115" s="4"/>
+      <x:c r="N115" s="5"/>
+    </x:row>
+    <x:row r="116" ht="24" customHeight="1">
+      <x:c r="A116" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B116" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C116" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_55</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D116" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E116" s="5"/>
+      <x:c r="F116" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G116" s="4"/>
+      <x:c r="H116" s="6"/>
+      <x:c r="I116" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J116" s="0"/>
+      <x:c r="K116" s="4"/>
+      <x:c r="L116" s="4"/>
+      <x:c r="M116" s="4"/>
+      <x:c r="N116" s="5"/>
+    </x:row>
+    <x:row r="117" ht="24" customHeight="1">
+      <x:c r="A117" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B117" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C117" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D117" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E117" s="5"/>
+      <x:c r="F117" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G117" s="4"/>
+      <x:c r="H117" s="6"/>
+      <x:c r="I117" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J117" s="0"/>
+      <x:c r="K117" s="4"/>
+      <x:c r="L117" s="4"/>
+      <x:c r="M117" s="4"/>
+      <x:c r="N117" s="5"/>
+    </x:row>
+    <x:row r="118" ht="24" customHeight="1">
+      <x:c r="A118" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B118" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C118" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D118" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E118" s="5"/>
+      <x:c r="F118" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G118" s="4"/>
+      <x:c r="H118" s="6"/>
+      <x:c r="I118" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J118" s="0"/>
+      <x:c r="K118" s="4"/>
+      <x:c r="L118" s="4"/>
+      <x:c r="M118" s="4"/>
+      <x:c r="N118" s="5"/>
+    </x:row>
+    <x:row r="119" ht="24" customHeight="1">
+      <x:c r="A119" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B119" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C119" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D119" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E119" s="5">
+        <x:v>0.8452</x:v>
+      </x:c>
+      <x:c r="F119" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G119" s="4"/>
+      <x:c r="H119" s="6"/>
+      <x:c r="I119" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J119" s="0">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="K119" s="4">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="L119" s="4">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="M119" s="4">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="N119" s="5">
+        <x:v>0.7115</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120" ht="24" customHeight="1">
+      <x:c r="A120" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B120" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C120" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D120" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E120" s="5"/>
+      <x:c r="F120" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G120" s="4"/>
+      <x:c r="H120" s="6"/>
+      <x:c r="I120" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J120" s="0"/>
+      <x:c r="K120" s="4"/>
+      <x:c r="L120" s="4"/>
+      <x:c r="M120" s="4"/>
+      <x:c r="N120" s="5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Gemini: add test results for Closure (54-79, count: 24)
</commit_message>
<xml_diff>
--- a/Gemini-3.8-flash/summary.xlsx
+++ b/Gemini-3.8-flash/summary.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N120" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ResultsData" displayName="ResultsData" ref="A1:N144" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="row_type"/>
     <x:tableColumn id="2" name="round"/>
@@ -412,16 +412,16 @@
         <x:v>Results</x:v>
       </x:c>
       <x:c r="C6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$120,"Round1")</x:f>
-        <x:v>119</x:v>
+        <x:f>COUNTIF(Data!$B$2:$B$144,"Round1")</x:f>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="D6" s="10">
-        <x:f>COUNTIF(Data!$B$2:$B$120,"Round2")</x:f>
+        <x:f>COUNTIF(Data!$B$2:$B$144,"Round2")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="11">
-        <x:f>COUNTA(Data!$C$2:$C$120)</x:f>
-        <x:v>119</x:v>
+        <x:f>COUNTA(Data!$C$2:$C$144)</x:f>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
@@ -435,16 +435,16 @@
         <x:v>Average line coverage</x:v>
       </x:c>
       <x:c r="C7" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$E$2:$E$120,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$120,"Round1",Data!$E$2:$E$120))</x:f>
-        <x:v>0.37134821428571435</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$E$2:$E$144,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$144,"Round1",Data!$E$2:$E$144))</x:f>
+        <x:v>0.38237719298245615</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$E$2:$E$120,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$120,"Round2",Data!$E$2:$E$120))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$E$2:$E$144,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$144,"Round2",Data!$E$2:$E$144))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E7" s="12">
-        <x:f>IF(COUNT(Data!$E$2:$E$120)=0,"",AVERAGE(Data!$E$2:$E$120))</x:f>
-        <x:v>0.37134821428571435</x:v>
+        <x:f>IF(COUNT(Data!$E$2:$E$144)=0,"",AVERAGE(Data!$E$2:$E$144))</x:f>
+        <x:v>0.38237719298245615</x:v>
       </x:c>
       <x:c r="F7" s="1"/>
       <x:c r="G7" s="1"/>
@@ -460,16 +460,16 @@
         </x:is>
       </x:c>
       <x:c r="C8" s="5">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$N$2:$N$120,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$120,"Round1",Data!$N$2:$N$120))</x:f>
-        <x:v>0.31776</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$N$2:$N$144,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$144,"Round1",Data!$N$2:$N$144))</x:f>
+        <x:v>0.32994285714285715</x:v>
       </x:c>
       <x:c r="D8" s="5" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$N$2:$N$120,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$120,"Round2",Data!$N$2:$N$120))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$N$2:$N$144,"&lt;&gt;")=0,"",AVERAGEIF(Data!$B$2:$B$144,"Round2",Data!$N$2:$N$144))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E8" s="12">
-        <x:f>IF(COUNT(Data!$N$2:$N$120)=0,"",AVERAGE(Data!$N$2:$N$120))</x:f>
-        <x:v>0.31776</x:v>
+        <x:f>IF(COUNT(Data!$N$2:$N$144)=0,"",AVERAGE(Data!$N$2:$N$144))</x:f>
+        <x:v>0.32994285714285715</x:v>
       </x:c>
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
@@ -483,15 +483,15 @@
         <x:v>Revealing results</x:v>
       </x:c>
       <x:c r="C9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$120,"Round1",Data!$F$2:$F$120)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$144,"Round1",Data!$F$2:$F$144)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="10">
-        <x:f>SUMIF(Data!$B$2:$B$120,"Round2",Data!$F$2:$F$120)</x:f>
+        <x:f>SUMIF(Data!$B$2:$B$144,"Round2",Data!$F$2:$F$144)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="11">
-        <x:f>SUM(Data!$F$2:$F$120)</x:f>
+        <x:f>SUM(Data!$F$2:$F$144)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="1"/>
@@ -529,16 +529,16 @@
         <x:v>Total tokens</x:v>
       </x:c>
       <x:c r="C11" s="10">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$G$2:$G$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$G$2:$G$120))</x:f>
-        <x:v>861110</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$G$2:$G$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round1",Data!$G$2:$G$144))</x:f>
+        <x:v>866010</x:v>
       </x:c>
       <x:c r="D11" s="10" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$G$2:$G$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$G$2:$G$120))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$G$2:$G$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round2",Data!$G$2:$G$144))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E11" s="11">
-        <x:f>IF(COUNT(Data!$G$2:$G$120)=0,"",SUM(Data!$G$2:$G$120))</x:f>
-        <x:v>861110</x:v>
+        <x:f>IF(COUNT(Data!$G$2:$G$144)=0,"",SUM(Data!$G$2:$G$144))</x:f>
+        <x:v>866010</x:v>
       </x:c>
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
@@ -552,16 +552,16 @@
         <x:v>Generation time (seconds)</x:v>
       </x:c>
       <x:c r="C12" s="6">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$H$2:$H$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$H$2:$H$120))</x:f>
-        <x:v>3425.85</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$H$2:$H$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round1",Data!$H$2:$H$144))</x:f>
+        <x:v>3440.6</x:v>
       </x:c>
       <x:c r="D12" s="6" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$H$2:$H$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$H$2:$H$120))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$H$2:$H$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round2",Data!$H$2:$H$144))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E12" s="13">
-        <x:f>IF(COUNT(Data!$H$2:$H$120)=0,"",SUM(Data!$H$2:$H$120))</x:f>
-        <x:v>3425.85</x:v>
+        <x:f>IF(COUNT(Data!$H$2:$H$144)=0,"",SUM(Data!$H$2:$H$144))</x:f>
+        <x:v>3440.6</x:v>
       </x:c>
       <x:c r="F12" s="1"/>
       <x:c r="G12" s="1"/>
@@ -575,16 +575,16 @@
         <x:v>Coverage records</x:v>
       </x:c>
       <x:c r="C13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$E$2:$E$120,"&lt;&gt;")</x:f>
-        <x:v>56</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$E$2:$E$144,"&lt;&gt;")</x:f>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D13" s="4">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$E$2:$E$120,"&lt;&gt;")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$E$2:$E$144,"&lt;&gt;")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E13" s="14">
-        <x:f>COUNT(Data!$E$2:$E$120)</x:f>
-        <x:v>56</x:v>
+        <x:f>COUNT(Data!$E$2:$E$144)</x:f>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F13" s="1"/>
       <x:c r="G13" s="1"/>
@@ -600,16 +600,16 @@
         </x:is>
       </x:c>
       <x:c r="C14" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$J$2:$J$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$J$2:$J$120))</x:f>
-        <x:v>12942</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$J$2:$J$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round1",Data!$J$2:$J$144))</x:f>
+        <x:v>13016</x:v>
       </x:c>
       <x:c r="D14" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$J$2:$J$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$J$2:$J$120))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$J$2:$J$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round2",Data!$J$2:$J$144))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E14" s="4">
-        <x:f>IF(COUNT(Data!$J$2:$J$120)=0,"",SUM(Data!$J$2:$J$120))</x:f>
-        <x:v>12942</x:v>
+        <x:f>IF(COUNT(Data!$J$2:$J$144)=0,"",SUM(Data!$J$2:$J$144))</x:f>
+        <x:v>13016</x:v>
       </x:c>
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
@@ -625,16 +625,16 @@
         </x:is>
       </x:c>
       <x:c r="C15" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$K$2:$K$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$K$2:$K$120))</x:f>
-        <x:v>6081</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$K$2:$K$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round1",Data!$K$2:$K$144))</x:f>
+        <x:v>6155</x:v>
       </x:c>
       <x:c r="D15" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$K$2:$K$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$K$2:$K$120))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$K$2:$K$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round2",Data!$K$2:$K$144))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E15" s="4">
-        <x:f>IF(COUNT(Data!$K$2:$K$120)=0,"",SUM(Data!$K$2:$K$120))</x:f>
-        <x:v>6081</x:v>
+        <x:f>IF(COUNT(Data!$K$2:$K$144)=0,"",SUM(Data!$K$2:$K$144))</x:f>
+        <x:v>6155</x:v>
       </x:c>
       <x:c r="F15" s="1"/>
       <x:c r="G15" s="1"/>
@@ -650,16 +650,16 @@
         </x:is>
       </x:c>
       <x:c r="C16" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$L$2:$L$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$L$2:$L$120))</x:f>
-        <x:v>7132</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$L$2:$L$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round1",Data!$L$2:$L$144))</x:f>
+        <x:v>7164</x:v>
       </x:c>
       <x:c r="D16" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$L$2:$L$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$L$2:$L$120))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$L$2:$L$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round2",Data!$L$2:$L$144))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E16" s="4">
-        <x:f>IF(COUNT(Data!$L$2:$L$120)=0,"",SUM(Data!$L$2:$L$120))</x:f>
-        <x:v>7132</x:v>
+        <x:f>IF(COUNT(Data!$L$2:$L$144)=0,"",SUM(Data!$L$2:$L$144))</x:f>
+        <x:v>7164</x:v>
       </x:c>
       <x:c r="F16" s="1"/>
       <x:c r="G16" s="1"/>
@@ -675,16 +675,16 @@
         </x:is>
       </x:c>
       <x:c r="C17" s="4">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$M$2:$M$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round1",Data!$M$2:$M$120))</x:f>
-        <x:v>2539</x:v>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$M$2:$M$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round1",Data!$M$2:$M$144))</x:f>
+        <x:v>2571</x:v>
       </x:c>
       <x:c r="D17" s="4" t="str">
-        <x:f>IF(COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$M$2:$M$120,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$120,"Round2",Data!$M$2:$M$120))</x:f>
+        <x:f>IF(COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$M$2:$M$144,"&lt;&gt;")=0,"",SUMIF(Data!$B$2:$B$144,"Round2",Data!$M$2:$M$144))</x:f>
         <x:v/>
       </x:c>
       <x:c r="E17" s="4">
-        <x:f>IF(COUNT(Data!$M$2:$M$120)=0,"",SUM(Data!$M$2:$M$120))</x:f>
-        <x:v>2539</x:v>
+        <x:f>IF(COUNT(Data!$M$2:$M$144)=0,"",SUM(Data!$M$2:$M$144))</x:f>
+        <x:v>2571</x:v>
       </x:c>
       <x:c r="F17" s="1"/>
       <x:c r="G17" s="1"/>
@@ -718,15 +718,15 @@
         <x:v>REVEALING</x:v>
       </x:c>
       <x:c r="C19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$D$2:$D$120,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$D$2:$D$144,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D19" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$D$2:$D$120,"REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$D$2:$D$144,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E19" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$120,"REVEALING")</x:f>
+        <x:f>COUNTIF(Data!$D$2:$D$144,"REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="1"/>
@@ -741,15 +741,15 @@
         <x:v>NOT_REVEALING</x:v>
       </x:c>
       <x:c r="C20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$D$2:$D$120,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$D$2:$D$144,"NOT_REVEALING")</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="D20" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$D$2:$D$120,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$D$2:$D$144,"NOT_REVEALING")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E20" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$120,"NOT_REVEALING")</x:f>
+        <x:f>COUNTIF(Data!$D$2:$D$144,"NOT_REVEALING")</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="F20" s="1"/>
@@ -764,16 +764,16 @@
         <x:v>NOT_AVAILABLE</x:v>
       </x:c>
       <x:c r="C21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$D$2:$D$120,"NOT_AVAILABLE")</x:f>
-        <x:v>64</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$D$2:$D$144,"NOT_AVAILABLE")</x:f>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="D21" s="9">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$D$2:$D$120,"NOT_AVAILABLE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$D$2:$D$144,"NOT_AVAILABLE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E21" s="9">
-        <x:f>COUNTIF(Data!$D$2:$D$120,"NOT_AVAILABLE")</x:f>
-        <x:v>64</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$144,"NOT_AVAILABLE")</x:f>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="F21" s="1"/>
       <x:c r="G21" s="1"/>
@@ -787,16 +787,16 @@
         <x:v>INCONCLUSIVE</x:v>
       </x:c>
       <x:c r="C22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round1",Data!$D$2:$D$120,"INCONCLUSIVE")</x:f>
-        <x:v>40</x:v>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round1",Data!$D$2:$D$144,"INCONCLUSIVE")</x:f>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D22" s="1">
-        <x:f>COUNTIFS(Data!$B$2:$B$120,"Round2",Data!$D$2:$D$120,"INCONCLUSIVE")</x:f>
+        <x:f>COUNTIFS(Data!$B$2:$B$144,"Round2",Data!$D$2:$D$144,"INCONCLUSIVE")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E22" s="1">
-        <x:f>COUNTIF(Data!$D$2:$D$120,"INCONCLUSIVE")</x:f>
-        <x:v>40</x:v>
+        <x:f>COUNTIF(Data!$D$2:$D$144,"INCONCLUSIVE")</x:f>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="F22" s="1"/>
       <x:c r="G22" s="1"/>
@@ -836,7 +836,7 @@
       <x:c r="A25" s="1"/>
       <x:c r="B25" s="3" t="inlineStr">
         <x:is>
-          <x:t>Updated: 2026-09-30 05:45:10 +0700</x:t>
+          <x:t>Updated: 2026-09-30 05:51:21 +0700</x:t>
         </x:is>
       </x:c>
       <x:c r="C25" s="3"/>
@@ -6014,7 +6014,7 @@
       </x:c>
       <x:c r="C116" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_55</x:t>
+          <x:t>Closure_54</x:t>
         </x:is>
       </x:c>
       <x:c r="D116" s="1" t="inlineStr">
@@ -6050,7 +6050,7 @@
       </x:c>
       <x:c r="C117" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_6</x:t>
+          <x:t>Closure_55</x:t>
         </x:is>
       </x:c>
       <x:c r="D117" s="1" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </x:c>
       <x:c r="C118" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_7</x:t>
+          <x:t>Closure_56</x:t>
         </x:is>
       </x:c>
       <x:c r="D118" s="1" t="inlineStr">
@@ -6122,17 +6122,15 @@
       </x:c>
       <x:c r="C119" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_8</x:t>
+          <x:t>Closure_57</x:t>
         </x:is>
       </x:c>
       <x:c r="D119" s="1" t="inlineStr">
         <x:is>
-          <x:t>INCONCLUSIVE</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E119" s="5">
-        <x:v>0.8452</x:v>
-      </x:c>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E119" s="5"/>
       <x:c r="F119" s="4">
         <x:v>0</x:v>
       </x:c>
@@ -6141,21 +6139,11 @@
       <x:c r="I119" s="16">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J119" s="0">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="K119" s="4">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="L119" s="4">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="M119" s="4">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="N119" s="5">
-        <x:v>0.7115</x:v>
-      </x:c>
+      <x:c r="J119" s="0"/>
+      <x:c r="K119" s="4"/>
+      <x:c r="L119" s="4"/>
+      <x:c r="M119" s="4"/>
+      <x:c r="N119" s="5"/>
     </x:row>
     <x:row r="120" ht="24" customHeight="1">
       <x:c r="A120" s="1" t="inlineStr">
@@ -6170,7 +6158,7 @@
       </x:c>
       <x:c r="C120" s="1" t="inlineStr">
         <x:is>
-          <x:t>Closure_9</x:t>
+          <x:t>Closure_58</x:t>
         </x:is>
       </x:c>
       <x:c r="D120" s="1" t="inlineStr">
@@ -6192,6 +6180,898 @@
       <x:c r="L120" s="4"/>
       <x:c r="M120" s="4"/>
       <x:c r="N120" s="5"/>
+    </x:row>
+    <x:row r="121" ht="24" customHeight="1">
+      <x:c r="A121" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B121" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C121" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_59</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D121" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E121" s="5"/>
+      <x:c r="F121" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G121" s="4"/>
+      <x:c r="H121" s="6"/>
+      <x:c r="I121" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J121" s="0"/>
+      <x:c r="K121" s="4"/>
+      <x:c r="L121" s="4"/>
+      <x:c r="M121" s="4"/>
+      <x:c r="N121" s="5"/>
+    </x:row>
+    <x:row r="122" ht="24" customHeight="1">
+      <x:c r="A122" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B122" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C122" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D122" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E122" s="5"/>
+      <x:c r="F122" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G122" s="4"/>
+      <x:c r="H122" s="6"/>
+      <x:c r="I122" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J122" s="0"/>
+      <x:c r="K122" s="4"/>
+      <x:c r="L122" s="4"/>
+      <x:c r="M122" s="4"/>
+      <x:c r="N122" s="5"/>
+    </x:row>
+    <x:row r="123" ht="24" customHeight="1">
+      <x:c r="A123" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B123" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C123" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_60</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D123" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E123" s="5"/>
+      <x:c r="F123" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G123" s="4"/>
+      <x:c r="H123" s="6"/>
+      <x:c r="I123" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J123" s="0"/>
+      <x:c r="K123" s="4"/>
+      <x:c r="L123" s="4"/>
+      <x:c r="M123" s="4"/>
+      <x:c r="N123" s="5"/>
+    </x:row>
+    <x:row r="124" ht="24" customHeight="1">
+      <x:c r="A124" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B124" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C124" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_61</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D124" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E124" s="5"/>
+      <x:c r="F124" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G124" s="4"/>
+      <x:c r="H124" s="6"/>
+      <x:c r="I124" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J124" s="0"/>
+      <x:c r="K124" s="4"/>
+      <x:c r="L124" s="4"/>
+      <x:c r="M124" s="4"/>
+      <x:c r="N124" s="5"/>
+    </x:row>
+    <x:row r="125" ht="24" customHeight="1">
+      <x:c r="A125" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B125" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C125" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D125" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E125" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+      <x:c r="F125" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G125" s="4">
+        <x:v>4900</x:v>
+      </x:c>
+      <x:c r="H125" s="6">
+        <x:v>14.75</x:v>
+      </x:c>
+      <x:c r="I125" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J125" s="0">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="K125" s="4">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="L125" s="4">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="M125" s="4">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="N125" s="5">
+        <x:v>1.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126" ht="24" customHeight="1">
+      <x:c r="A126" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B126" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C126" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_64</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D126" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E126" s="5"/>
+      <x:c r="F126" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G126" s="4"/>
+      <x:c r="H126" s="6"/>
+      <x:c r="I126" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J126" s="0"/>
+      <x:c r="K126" s="4"/>
+      <x:c r="L126" s="4"/>
+      <x:c r="M126" s="4"/>
+      <x:c r="N126" s="5"/>
+    </x:row>
+    <x:row r="127" ht="24" customHeight="1">
+      <x:c r="A127" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B127" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C127" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_65</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D127" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E127" s="5"/>
+      <x:c r="F127" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G127" s="4"/>
+      <x:c r="H127" s="6"/>
+      <x:c r="I127" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J127" s="0"/>
+      <x:c r="K127" s="4"/>
+      <x:c r="L127" s="4"/>
+      <x:c r="M127" s="4"/>
+      <x:c r="N127" s="5"/>
+    </x:row>
+    <x:row r="128" ht="24" customHeight="1">
+      <x:c r="A128" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B128" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C128" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_66</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D128" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E128" s="5"/>
+      <x:c r="F128" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G128" s="4"/>
+      <x:c r="H128" s="6"/>
+      <x:c r="I128" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J128" s="0"/>
+      <x:c r="K128" s="4"/>
+      <x:c r="L128" s="4"/>
+      <x:c r="M128" s="4"/>
+      <x:c r="N128" s="5"/>
+    </x:row>
+    <x:row r="129" ht="24" customHeight="1">
+      <x:c r="A129" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B129" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C129" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D129" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E129" s="5"/>
+      <x:c r="F129" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G129" s="4"/>
+      <x:c r="H129" s="6"/>
+      <x:c r="I129" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J129" s="0"/>
+      <x:c r="K129" s="4"/>
+      <x:c r="L129" s="4"/>
+      <x:c r="M129" s="4"/>
+      <x:c r="N129" s="5"/>
+    </x:row>
+    <x:row r="130" ht="24" customHeight="1">
+      <x:c r="A130" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B130" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C130" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D130" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E130" s="5"/>
+      <x:c r="F130" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G130" s="4"/>
+      <x:c r="H130" s="6"/>
+      <x:c r="I130" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J130" s="0"/>
+      <x:c r="K130" s="4"/>
+      <x:c r="L130" s="4"/>
+      <x:c r="M130" s="4"/>
+      <x:c r="N130" s="5"/>
+    </x:row>
+    <x:row r="131" ht="24" customHeight="1">
+      <x:c r="A131" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B131" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C131" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_69</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D131" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E131" s="5"/>
+      <x:c r="F131" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G131" s="4"/>
+      <x:c r="H131" s="6"/>
+      <x:c r="I131" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J131" s="0"/>
+      <x:c r="K131" s="4"/>
+      <x:c r="L131" s="4"/>
+      <x:c r="M131" s="4"/>
+      <x:c r="N131" s="5"/>
+    </x:row>
+    <x:row r="132" ht="24" customHeight="1">
+      <x:c r="A132" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B132" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C132" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D132" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E132" s="5"/>
+      <x:c r="F132" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G132" s="4"/>
+      <x:c r="H132" s="6"/>
+      <x:c r="I132" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J132" s="0"/>
+      <x:c r="K132" s="4"/>
+      <x:c r="L132" s="4"/>
+      <x:c r="M132" s="4"/>
+      <x:c r="N132" s="5"/>
+    </x:row>
+    <x:row r="133" ht="24" customHeight="1">
+      <x:c r="A133" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B133" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C133" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_70</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D133" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E133" s="5"/>
+      <x:c r="F133" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G133" s="4"/>
+      <x:c r="H133" s="6"/>
+      <x:c r="I133" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J133" s="0"/>
+      <x:c r="K133" s="4"/>
+      <x:c r="L133" s="4"/>
+      <x:c r="M133" s="4"/>
+      <x:c r="N133" s="5"/>
+    </x:row>
+    <x:row r="134" ht="24" customHeight="1">
+      <x:c r="A134" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B134" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C134" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_71</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D134" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E134" s="5"/>
+      <x:c r="F134" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G134" s="4"/>
+      <x:c r="H134" s="6"/>
+      <x:c r="I134" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J134" s="0"/>
+      <x:c r="K134" s="4"/>
+      <x:c r="L134" s="4"/>
+      <x:c r="M134" s="4"/>
+      <x:c r="N134" s="5"/>
+    </x:row>
+    <x:row r="135" ht="24" customHeight="1">
+      <x:c r="A135" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B135" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C135" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_72</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D135" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E135" s="5"/>
+      <x:c r="F135" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G135" s="4"/>
+      <x:c r="H135" s="6"/>
+      <x:c r="I135" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J135" s="0"/>
+      <x:c r="K135" s="4"/>
+      <x:c r="L135" s="4"/>
+      <x:c r="M135" s="4"/>
+      <x:c r="N135" s="5"/>
+    </x:row>
+    <x:row r="136" ht="24" customHeight="1">
+      <x:c r="A136" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B136" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C136" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_73</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D136" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E136" s="5"/>
+      <x:c r="F136" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G136" s="4"/>
+      <x:c r="H136" s="6"/>
+      <x:c r="I136" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J136" s="0"/>
+      <x:c r="K136" s="4"/>
+      <x:c r="L136" s="4"/>
+      <x:c r="M136" s="4"/>
+      <x:c r="N136" s="5"/>
+    </x:row>
+    <x:row r="137" ht="24" customHeight="1">
+      <x:c r="A137" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B137" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C137" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_74</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D137" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E137" s="5"/>
+      <x:c r="F137" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G137" s="4"/>
+      <x:c r="H137" s="6"/>
+      <x:c r="I137" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J137" s="0"/>
+      <x:c r="K137" s="4"/>
+      <x:c r="L137" s="4"/>
+      <x:c r="M137" s="4"/>
+      <x:c r="N137" s="5"/>
+    </x:row>
+    <x:row r="138" ht="24" customHeight="1">
+      <x:c r="A138" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B138" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C138" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_75</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D138" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E138" s="5"/>
+      <x:c r="F138" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G138" s="4"/>
+      <x:c r="H138" s="6"/>
+      <x:c r="I138" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J138" s="0"/>
+      <x:c r="K138" s="4"/>
+      <x:c r="L138" s="4"/>
+      <x:c r="M138" s="4"/>
+      <x:c r="N138" s="5"/>
+    </x:row>
+    <x:row r="139" ht="24" customHeight="1">
+      <x:c r="A139" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B139" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C139" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_76</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D139" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E139" s="5"/>
+      <x:c r="F139" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G139" s="4"/>
+      <x:c r="H139" s="6"/>
+      <x:c r="I139" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J139" s="0"/>
+      <x:c r="K139" s="4"/>
+      <x:c r="L139" s="4"/>
+      <x:c r="M139" s="4"/>
+      <x:c r="N139" s="5"/>
+    </x:row>
+    <x:row r="140" ht="24" customHeight="1">
+      <x:c r="A140" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B140" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C140" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_77</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D140" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E140" s="5"/>
+      <x:c r="F140" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G140" s="4"/>
+      <x:c r="H140" s="6"/>
+      <x:c r="I140" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J140" s="0"/>
+      <x:c r="K140" s="4"/>
+      <x:c r="L140" s="4"/>
+      <x:c r="M140" s="4"/>
+      <x:c r="N140" s="5"/>
+    </x:row>
+    <x:row r="141" ht="24" customHeight="1">
+      <x:c r="A141" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B141" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C141" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_78</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D141" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E141" s="5"/>
+      <x:c r="F141" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G141" s="4"/>
+      <x:c r="H141" s="6"/>
+      <x:c r="I141" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J141" s="0"/>
+      <x:c r="K141" s="4"/>
+      <x:c r="L141" s="4"/>
+      <x:c r="M141" s="4"/>
+      <x:c r="N141" s="5"/>
+    </x:row>
+    <x:row r="142" ht="24" customHeight="1">
+      <x:c r="A142" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B142" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C142" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_79</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D142" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E142" s="5"/>
+      <x:c r="F142" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G142" s="4"/>
+      <x:c r="H142" s="6"/>
+      <x:c r="I142" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J142" s="0"/>
+      <x:c r="K142" s="4"/>
+      <x:c r="L142" s="4"/>
+      <x:c r="M142" s="4"/>
+      <x:c r="N142" s="5"/>
+    </x:row>
+    <x:row r="143" ht="24" customHeight="1">
+      <x:c r="A143" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B143" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C143" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D143" s="1" t="inlineStr">
+        <x:is>
+          <x:t>INCONCLUSIVE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E143" s="5">
+        <x:v>0.8452</x:v>
+      </x:c>
+      <x:c r="F143" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G143" s="4"/>
+      <x:c r="H143" s="6"/>
+      <x:c r="I143" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J143" s="0">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="K143" s="4">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="L143" s="4">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="M143" s="4">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="N143" s="5">
+        <x:v>0.7115</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144" ht="24" customHeight="1">
+      <x:c r="A144" s="1" t="inlineStr">
+        <x:is>
+          <x:t>RESULT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B144" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Round1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C144" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Closure_9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D144" s="1" t="inlineStr">
+        <x:is>
+          <x:t>NOT_AVAILABLE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E144" s="5"/>
+      <x:c r="F144" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G144" s="4"/>
+      <x:c r="H144" s="6"/>
+      <x:c r="I144" s="16">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J144" s="0"/>
+      <x:c r="K144" s="4"/>
+      <x:c r="L144" s="4"/>
+      <x:c r="M144" s="4"/>
+      <x:c r="N144" s="5"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>